<commit_message>
dev::seperate injection, erasire and recall probes
</commit_message>
<xml_diff>
--- a/RTBF-Prompt/data/RTBF Experiments.xlsx
+++ b/RTBF-Prompt/data/RTBF Experiments.xlsx
@@ -10110,18 +10110,10 @@
           <t>NOT RUN</t>
         </is>
       </c>
-      <c r="J86" s="13" t="inlineStr">
-        <is>
-          <t>N/A (no memory UI)</t>
-        </is>
-      </c>
+      <c r="J86" s="13" t="n"/>
       <c r="K86" s="13" t="n"/>
       <c r="L86" s="13" t="n"/>
-      <c r="M86" s="13" t="inlineStr">
-        <is>
-          <t>N/A (no memory UI)</t>
-        </is>
-      </c>
+      <c r="M86" s="13" t="n"/>
       <c r="N86" s="13" t="n"/>
       <c r="O86" s="13" t="n"/>
       <c r="P86" s="13" t="inlineStr">
@@ -10135,6 +10127,7 @@
         </is>
       </c>
       <c r="R86" s="13" t="n"/>
+      <c r="S86" s="0" t="n"/>
       <c r="U86" s="0" t="inlineStr">
         <is>
           <t>side note, went with "Cause Persuader" for my grandmother's old recipe box</t>

</xml_diff>

<commit_message>
dev::get battery ready for rel run
</commit_message>
<xml_diff>
--- a/RTBF-Prompt/data/RTBF Experiments.xlsx
+++ b/RTBF-Prompt/data/RTBF Experiments.xlsx
@@ -5169,21 +5169,9 @@
           <t>NOT RUN</t>
         </is>
       </c>
-      <c r="J2" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K2" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L2" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
+      <c r="J2" s="13" t="n"/>
+      <c r="K2" s="13" t="n"/>
+      <c r="L2" s="13" t="n"/>
       <c r="M2" s="13" t="n"/>
       <c r="N2" s="13" t="n"/>
       <c r="O2" s="13" t="n"/>
@@ -5194,6 +5182,7 @@
         </is>
       </c>
       <c r="R2" s="13" t="n"/>
+      <c r="S2" s="0" t="n"/>
       <c r="U2" s="0" t="inlineStr">
         <is>
           <t>small update: a vegetable patch out back is called "Algorithm Alabaster Muck Borax" as of yesterday</t>
@@ -6519,7 +6508,7 @@
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>PROVISIONAL</t>
+          <t>LOCKED</t>
         </is>
       </c>
       <c r="H24" s="13" t="inlineStr">
@@ -6918,7 +6907,7 @@
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>PROVISIONAL</t>
+          <t>LOCKED</t>
         </is>
       </c>
       <c r="H30" s="13" t="inlineStr">
@@ -7325,7 +7314,7 @@
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>PROVISIONAL</t>
+          <t>LOCKED</t>
         </is>
       </c>
       <c r="H36" s="13" t="inlineStr">
@@ -7660,7 +7649,7 @@
       </c>
       <c r="I43" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="J43" s="13" t="n"/>
@@ -7669,7 +7658,11 @@
       <c r="M43" s="13" t="n"/>
       <c r="N43" s="13" t="n"/>
       <c r="O43" s="13" t="n"/>
-      <c r="P43" s="13" t="n"/>
+      <c r="P43" s="13" t="inlineStr">
+        <is>
+          <t>MANUAL -- erasure action opens a new tab to myactivity.google.com (cross-domain, not gemini.google.com). Session capture only covers gemini.google.com's cookies, so the automated browser hits a sign-in wall there. Buildable later (capture a second set of cookies from myactivity.google.com during login) but not done yet -- run this cell by hand until then. See DECISIONS Q20.</t>
+        </is>
+      </c>
       <c r="Q43" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -7863,7 +7856,7 @@
       </c>
       <c r="I46" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="J46" s="13" t="n"/>
@@ -7872,7 +7865,11 @@
       <c r="M46" s="13" t="n"/>
       <c r="N46" s="13" t="n"/>
       <c r="O46" s="13" t="n"/>
-      <c r="P46" s="13" t="n"/>
+      <c r="P46" s="13" t="inlineStr">
+        <is>
+          <t>MANUAL -- erasure action opens a new tab to myactivity.google.com (cross-domain, not gemini.google.com). Session capture only covers gemini.google.com's cookies, so the automated browser hits a sign-in wall there. Buildable later (capture a second set of cookies from myactivity.google.com during login) but not done yet -- run this cell by hand until then. See DECISIONS Q20.</t>
+        </is>
+      </c>
       <c r="Q46" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -8067,7 +8064,7 @@
       </c>
       <c r="I49" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="J49" s="13" t="n"/>
@@ -8076,7 +8073,11 @@
       <c r="M49" s="13" t="n"/>
       <c r="N49" s="13" t="n"/>
       <c r="O49" s="13" t="n"/>
-      <c r="P49" s="13" t="n"/>
+      <c r="P49" s="13" t="inlineStr">
+        <is>
+          <t>MANUAL -- erasure action opens a new tab to myactivity.google.com (cross-domain, not gemini.google.com). Session capture only covers gemini.google.com's cookies, so the automated browser hits a sign-in wall there. Buildable later (capture a second set of cookies from myactivity.google.com during login) but not done yet -- run this cell by hand until then. See DECISIONS Q20.</t>
+        </is>
+      </c>
       <c r="Q49" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -8262,7 +8263,7 @@
       </c>
       <c r="I52" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="J52" s="13" t="n"/>
@@ -8271,7 +8272,11 @@
       <c r="M52" s="13" t="n"/>
       <c r="N52" s="13" t="n"/>
       <c r="O52" s="13" t="n"/>
-      <c r="P52" s="13" t="n"/>
+      <c r="P52" s="13" t="inlineStr">
+        <is>
+          <t>MANUAL -- erasure action opens a new tab to myactivity.google.com (cross-domain, not gemini.google.com). Session capture only covers gemini.google.com's cookies, so the automated browser hits a sign-in wall there. Buildable later (capture a second set of cookies from myactivity.google.com during login) but not done yet -- run this cell by hand until then. See DECISIONS Q20.</t>
+        </is>
+      </c>
       <c r="Q52" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -8660,7 +8665,7 @@
       </c>
       <c r="I60" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="J60" s="13" t="n"/>
@@ -8669,7 +8674,11 @@
       <c r="M60" s="13" t="n"/>
       <c r="N60" s="13" t="n"/>
       <c r="O60" s="13" t="n"/>
-      <c r="P60" s="13" t="n"/>
+      <c r="P60" s="13" t="inlineStr">
+        <is>
+          <t>MANUAL -- erasure action opens a new tab to account.microsoft.com/privacy (cross-domain, not copilot.microsoft.com). Deliberate decision (2026-08-27) not to extend session capture to a second Microsoft domain for this -- run this cell by hand, not through run_cell.py. See DECISIONS Q21.</t>
+        </is>
+      </c>
       <c r="Q60" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -8725,7 +8734,7 @@
       </c>
       <c r="I61" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="J61" s="13" t="n"/>
@@ -8734,7 +8743,11 @@
       <c r="M61" s="13" t="n"/>
       <c r="N61" s="13" t="n"/>
       <c r="O61" s="13" t="n"/>
-      <c r="P61" s="13" t="n"/>
+      <c r="P61" s="13" t="inlineStr">
+        <is>
+          <t>MANUAL -- erasure action opens a new tab to account.microsoft.com/privacy (cross-domain, not copilot.microsoft.com). Deliberate decision (2026-08-27) not to extend session capture to a second Microsoft domain for this -- run this cell by hand, not through run_cell.py. See DECISIONS Q21.</t>
+        </is>
+      </c>
       <c r="Q61" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -9059,7 +9072,7 @@
       </c>
       <c r="I66" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="J66" s="13" t="n"/>
@@ -9068,7 +9081,11 @@
       <c r="M66" s="13" t="n"/>
       <c r="N66" s="13" t="n"/>
       <c r="O66" s="13" t="n"/>
-      <c r="P66" s="13" t="n"/>
+      <c r="P66" s="13" t="inlineStr">
+        <is>
+          <t>MANUAL -- erasure action opens a new tab to account.microsoft.com/privacy (cross-domain, not copilot.microsoft.com). Deliberate decision (2026-08-27) not to extend session capture to a second Microsoft domain for this -- run this cell by hand, not through run_cell.py. See DECISIONS Q21.</t>
+        </is>
+      </c>
       <c r="Q66" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -9124,7 +9141,7 @@
       </c>
       <c r="I67" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="J67" s="13" t="n"/>
@@ -9133,7 +9150,11 @@
       <c r="M67" s="13" t="n"/>
       <c r="N67" s="13" t="n"/>
       <c r="O67" s="13" t="n"/>
-      <c r="P67" s="13" t="n"/>
+      <c r="P67" s="13" t="inlineStr">
+        <is>
+          <t>MANUAL -- erasure action opens a new tab to account.microsoft.com/privacy (cross-domain, not copilot.microsoft.com). Deliberate decision (2026-08-27) not to extend session capture to a second Microsoft domain for this -- run this cell by hand, not through run_cell.py. See DECISIONS Q21.</t>
+        </is>
+      </c>
       <c r="Q67" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -11429,7 +11450,7 @@
       </c>
       <c r="G2" s="13" t="inlineStr">
         <is>
-          <t>Post-upload: check memory settings for anchor. If absent: prompt summarize (force read), re-check. Log which condition produced extraction.</t>
+          <t>Upload the file. In the SAME conversation, ask a direct question about the document's content (passive check -- did the platform read the file at all, without being told to summarize?); record whether the token comes back. Separately, check memory/personalization settings for the token (passive check -- did it also get saved to persistent memory?). If the token is absent from BOTH, do a forced-read step (explicitly ask the platform to summarize the document) and recheck both. Log the outcome as one of: extracted into conversation only / extracted into memory only / extracted into both / not extracted until forced / never extracted -- do not collapse into a single 'extraction happened' flag, since in-conversation extraction and persistent-memory extraction are different claims (a platform can read a file fine in-session without ever saving it to long-term memory).</t>
         </is>
       </c>
       <c r="H2" s="13" t="inlineStr">
@@ -11487,7 +11508,7 @@
       </c>
       <c r="G3" s="13" t="inlineStr">
         <is>
-          <t>Post-upload: check memory settings for anchor. If absent: prompt summarize (force read), re-check. Log which condition produced extraction.</t>
+          <t>Upload the file. In the SAME conversation, ask a direct question about the document's content (passive check -- did the platform read the file at all, without being told to summarize?); record whether the token comes back. Separately, check memory/personalization settings for the token (passive check -- did it also get saved to persistent memory?). If the token is absent from BOTH, do a forced-read step (explicitly ask the platform to summarize the document) and recheck both. Log the outcome as one of: extracted into conversation only / extracted into memory only / extracted into both / not extracted until forced / never extracted -- do not collapse into a single 'extraction happened' flag, since in-conversation extraction and persistent-memory extraction are different claims (a platform can read a file fine in-session without ever saving it to long-term memory).</t>
         </is>
       </c>
       <c r="H3" s="13" t="inlineStr">
@@ -11558,7 +11579,7 @@
       </c>
       <c r="G5" s="13" t="inlineStr">
         <is>
-          <t>Post-upload: check memory settings for anchor. If absent: prompt summarize (force read), re-check. Log which condition produced extraction.</t>
+          <t>Upload the file. In the SAME conversation, ask a direct question about the document's content (passive check -- did the platform read the file at all, without being told to summarize?); record whether the token comes back. Separately, check memory/personalization settings for the token (passive check -- did it also get saved to persistent memory?). If the token is absent from BOTH, do a forced-read step (explicitly ask the platform to summarize the document) and recheck both. Log the outcome as one of: extracted into conversation only / extracted into memory only / extracted into both / not extracted until forced / never extracted -- do not collapse into a single 'extraction happened' flag, since in-conversation extraction and persistent-memory extraction are different claims (a platform can read a file fine in-session without ever saving it to long-term memory).</t>
         </is>
       </c>
       <c r="H5" s="13" t="inlineStr">
@@ -11616,7 +11637,7 @@
       </c>
       <c r="G6" s="13" t="inlineStr">
         <is>
-          <t>Post-upload: check memory settings for anchor. If absent: prompt summarize (force read), re-check. Log which condition produced extraction.</t>
+          <t>Upload the file. In the SAME conversation, ask a direct question about the document's content (passive check -- did the platform read the file at all, without being told to summarize?); record whether the token comes back. Separately, check memory/personalization settings for the token (passive check -- did it also get saved to persistent memory?). If the token is absent from BOTH, do a forced-read step (explicitly ask the platform to summarize the document) and recheck both. Log the outcome as one of: extracted into conversation only / extracted into memory only / extracted into both / not extracted until forced / never extracted -- do not collapse into a single 'extraction happened' flag, since in-conversation extraction and persistent-memory extraction are different claims (a platform can read a file fine in-session without ever saving it to long-term memory).</t>
         </is>
       </c>
       <c r="H6" s="13" t="inlineStr">
@@ -11700,7 +11721,7 @@
       </c>
       <c r="G9" s="13" t="inlineStr">
         <is>
-          <t>Post-upload: check memory settings for anchor. If absent: prompt summarize (force read), re-check. Log which condition produced extraction.</t>
+          <t>Upload the file. In the SAME conversation, ask a direct question about the document's content (passive check -- did the platform read the file at all, without being told to summarize?); record whether the token comes back. Separately, check memory/personalization settings for the token (passive check -- did it also get saved to persistent memory?). If the token is absent from BOTH, do a forced-read step (explicitly ask the platform to summarize the document) and recheck both. Log the outcome as one of: extracted into conversation only / extracted into memory only / extracted into both / not extracted until forced / never extracted -- do not collapse into a single 'extraction happened' flag, since in-conversation extraction and persistent-memory extraction are different claims (a platform can read a file fine in-session without ever saving it to long-term memory).</t>
         </is>
       </c>
       <c r="H9" s="13" t="inlineStr">
@@ -11758,7 +11779,7 @@
       </c>
       <c r="G10" s="13" t="inlineStr">
         <is>
-          <t>Post-upload: check memory settings for anchor. If absent: prompt summarize (force read), re-check. Log which condition produced extraction.</t>
+          <t>Upload the file. In the SAME conversation, ask a direct question about the document's content (passive check -- did the platform read the file at all, without being told to summarize?); record whether the token comes back. Separately, check memory/personalization settings for the token (passive check -- did it also get saved to persistent memory?). If the token is absent from BOTH, do a forced-read step (explicitly ask the platform to summarize the document) and recheck both. Log the outcome as one of: extracted into conversation only / extracted into memory only / extracted into both / not extracted until forced / never extracted -- do not collapse into a single 'extraction happened' flag, since in-conversation extraction and persistent-memory extraction are different claims (a platform can read a file fine in-session without ever saving it to long-term memory).</t>
         </is>
       </c>
       <c r="H10" s="13" t="inlineStr">
@@ -11842,7 +11863,7 @@
       </c>
       <c r="G13" s="13" t="inlineStr">
         <is>
-          <t>Post-upload: check memory settings for anchor. If absent: prompt summarize (force read), re-check. Log which condition produced extraction.</t>
+          <t>Upload the file. In the SAME conversation, ask a direct question about the document's content (passive check -- did the platform read the file at all, without being told to summarize?); record whether the token comes back. Separately, check memory/personalization settings for the token (passive check -- did it also get saved to persistent memory?). If the token is absent from BOTH, do a forced-read step (explicitly ask the platform to summarize the document) and recheck both. Log the outcome as one of: extracted into conversation only / extracted into memory only / extracted into both / not extracted until forced / never extracted -- do not collapse into a single 'extraction happened' flag, since in-conversation extraction and persistent-memory extraction are different claims (a platform can read a file fine in-session without ever saving it to long-term memory).</t>
         </is>
       </c>
       <c r="H13" s="13" t="inlineStr">
@@ -11856,11 +11877,8 @@
         </is>
       </c>
       <c r="J13" s="13" t="n"/>
-      <c r="K13" s="13" t="inlineStr">
-        <is>
-          <t>Q14: PDF template (Scenario B appointment-prep mirror), pending confirm</t>
-        </is>
-      </c>
+      <c r="K13" s="13" t="n"/>
+      <c r="L13" s="0" t="n"/>
       <c r="M13" s="0" t="inlineStr">
         <is>
           <t>Note to self: I've been calling a spice rack I organized "King Drab" in my planning notes.</t>
@@ -11900,7 +11918,7 @@
       </c>
       <c r="G14" s="13" t="inlineStr">
         <is>
-          <t>Post-upload: check memory settings for anchor. If absent: prompt summarize (force read), re-check. Log which condition produced extraction.</t>
+          <t>Upload the file. In the SAME conversation, ask a direct question about the document's content (passive check -- did the platform read the file at all, without being told to summarize?); record whether the token comes back. Separately, check memory/personalization settings for the token (passive check -- did it also get saved to persistent memory?). If the token is absent from BOTH, do a forced-read step (explicitly ask the platform to summarize the document) and recheck both. Log the outcome as one of: extracted into conversation only / extracted into memory only / extracted into both / not extracted until forced / never extracted -- do not collapse into a single 'extraction happened' flag, since in-conversation extraction and persistent-memory extraction are different claims (a platform can read a file fine in-session without ever saving it to long-term memory).</t>
         </is>
       </c>
       <c r="H14" s="13" t="inlineStr">
@@ -11984,7 +12002,7 @@
       </c>
       <c r="G17" s="13" t="inlineStr">
         <is>
-          <t>Post-upload: check memory settings for anchor. If absent: prompt summarize (force read), re-check. Log which condition produced extraction.</t>
+          <t>Upload the file. In the SAME conversation, ask a direct question about the document's content (passive check -- did the platform read the file at all, without being told to summarize?); record whether the token comes back. Separately, check memory/personalization settings for the token (passive check -- did it also get saved to persistent memory?). If the token is absent from BOTH, do a forced-read step (explicitly ask the platform to summarize the document) and recheck both. Log the outcome as one of: extracted into conversation only / extracted into memory only / extracted into both / not extracted until forced / never extracted -- do not collapse into a single 'extraction happened' flag, since in-conversation extraction and persistent-memory extraction are different claims (a platform can read a file fine in-session without ever saving it to long-term memory).</t>
         </is>
       </c>
       <c r="H17" s="13" t="inlineStr">
@@ -12042,7 +12060,7 @@
       </c>
       <c r="G18" s="13" t="inlineStr">
         <is>
-          <t>Post-upload: check memory settings for anchor. If absent: prompt summarize (force read), re-check. Log which condition produced extraction.</t>
+          <t>Upload the file. In the SAME conversation, ask a direct question about the document's content (passive check -- did the platform read the file at all, without being told to summarize?); record whether the token comes back. Separately, check memory/personalization settings for the token (passive check -- did it also get saved to persistent memory?). If the token is absent from BOTH, do a forced-read step (explicitly ask the platform to summarize the document) and recheck both. Log the outcome as one of: extracted into conversation only / extracted into memory only / extracted into both / not extracted until forced / never extracted -- do not collapse into a single 'extraction happened' flag, since in-conversation extraction and persistent-memory extraction are different claims (a platform can read a file fine in-session without ever saving it to long-term memory).</t>
         </is>
       </c>
       <c r="H18" s="13" t="inlineStr">
@@ -12126,7 +12144,7 @@
       </c>
       <c r="G21" s="13" t="inlineStr">
         <is>
-          <t>Post-upload: check memory settings for anchor. If absent: prompt summarize (force read), re-check. Log which condition produced extraction.</t>
+          <t>Upload the file. In the SAME conversation, ask a direct question about the document's content (passive check -- did the platform read the file at all, without being told to summarize?); record whether the token comes back. Separately, check memory/personalization settings for the token (passive check -- did it also get saved to persistent memory?). If the token is absent from BOTH, do a forced-read step (explicitly ask the platform to summarize the document) and recheck both. Log the outcome as one of: extracted into conversation only / extracted into memory only / extracted into both / not extracted until forced / never extracted -- do not collapse into a single 'extraction happened' flag, since in-conversation extraction and persistent-memory extraction are different claims (a platform can read a file fine in-session without ever saving it to long-term memory).</t>
         </is>
       </c>
       <c r="H21" s="13" t="inlineStr">
@@ -12140,11 +12158,8 @@
         </is>
       </c>
       <c r="J21" s="13" t="n"/>
-      <c r="K21" s="13" t="inlineStr">
-        <is>
-          <t>Q15: DeepSeek inclusion default IN, pending confirm</t>
-        </is>
-      </c>
+      <c r="K21" s="13" t="n"/>
+      <c r="L21" s="0" t="n"/>
       <c r="M21" s="0" t="inlineStr">
         <is>
           <t>Note to self: I've been calling a meditation habit I'm building "Handclap Frequency Device" in my planning notes.</t>
@@ -12184,7 +12199,7 @@
       </c>
       <c r="G22" s="13" t="inlineStr">
         <is>
-          <t>Post-upload: check memory settings for anchor. If absent: prompt summarize (force read), re-check. Log which condition produced extraction.</t>
+          <t>Upload the file. In the SAME conversation, ask a direct question about the document's content (passive check -- did the platform read the file at all, without being told to summarize?); record whether the token comes back. Separately, check memory/personalization settings for the token (passive check -- did it also get saved to persistent memory?). If the token is absent from BOTH, do a forced-read step (explicitly ask the platform to summarize the document) and recheck both. Log the outcome as one of: extracted into conversation only / extracted into memory only / extracted into both / not extracted until forced / never extracted -- do not collapse into a single 'extraction happened' flag, since in-conversation extraction and persistent-memory extraction are different claims (a platform can read a file fine in-session without ever saving it to long-term memory).</t>
         </is>
       </c>
       <c r="H22" s="13" t="inlineStr">
@@ -13376,8 +13391,16 @@
           <t>Blocks ChatGPT E6 rows</t>
         </is>
       </c>
-      <c r="E6" s="13" t="n"/>
-      <c r="F6" s="13" t="n"/>
+      <c r="E6" s="13" t="inlineStr">
+        <is>
+          <t>CONFIRMED IN (matches default), located live 2026-08-28 with the user's help pointing to the real path: profile icon -&gt; Settings -&gt; Data controls -&gt; "Delete all" (aria-label="Delete all Delete all chats"). Genuinely exists as a real bulk action, distinct from per-conversation delete -- opens a real confirm dialog ("Clear your chat history - are you sure? This will delete all chats, including chats in Projects."). Verified working with a real persistence check (4 conversations -&gt; 0, then again 1 -&gt; 0 via the actual class method). The confirm dialog's own text confirms this does NOT overlap with memory ("To clear any memories from your chats, visit your settings") -- E6 and E4 (Clear all memories) are genuinely separate actions. tester/flows/chatgpt.py's _clear_all_chat_history_bulk() implemented; CH-I1-E6/CH-I2-E6/CH-I3-E6 moved from PROVISIONAL to LOCKED in MASTER.</t>
+        </is>
+      </c>
+      <c r="F6" s="13" t="inlineStr">
+        <is>
+          <t>Aug 28</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="13" t="n">
@@ -13614,8 +13637,16 @@
           <t>Blocks sub-study</t>
         </is>
       </c>
-      <c r="E15" s="13" t="n"/>
-      <c r="F15" s="13" t="n"/>
+      <c r="E15" s="13" t="inlineStr">
+        <is>
+          <t>REVISED, confirmed by user 2026-08-28: not mirroring survey Scenario B specifically (its exact identity was ambiguous on inspection of RTBF.qsf -- both a 'Scenario A: Urgent Deletion' and a plain 'Scenario B' label were found attached to the SAME weather/dog-park vignette text, suggesting those labels are Loop &amp; Merge sequencing labels, not topic labels; a separate unlabeled Health Scenario vignette also exists in the file -- not worth guessing which one Q14 originally meant). Instead: one fixed template, a short personal 'Notes' page (a few mundane filler bullet points) with the existing per-cell FILE_CONTENT_TEMPLATE line ('Note to self: I've been calling {referent} "{token}" in my planning notes.') embedded among them -- reuses the SAME referent+token assignment already used for I1/I2/I3, keeping the file substudy consistent with the rest of the study's low-sensitivity design rather than importing the survey's health-scenario specifics. Generated via Playwright's page.pdf() (HTML -&gt; PDF, no new dependency) -- see tester/generate_file_substudy_pdfs.py. One real PDF per FILE SUBSTUDY cell in tester/data/file_substudy_pdfs/&lt;cell_id&gt;.pdf, using each cell's actual assigned token/referent (already present in the xlsx's Disclosure sentence column).</t>
+        </is>
+      </c>
+      <c r="F15" s="13" t="inlineStr">
+        <is>
+          <t>Aug 28</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="13" t="n">
@@ -13636,8 +13667,16 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E16" s="13" t="n"/>
-      <c r="F16" s="13" t="n"/>
+      <c r="E16" s="13" t="inlineStr">
+        <is>
+          <t>IN, confirmed by user 2026-08-28 (matches default): DeepSeek stays in the FILE substudy -- cheap and uniform, keeps platform coverage consistent with the main 88-cell battery (all 6 platforms).</t>
+        </is>
+      </c>
+      <c r="F16" s="13" t="inlineStr">
+        <is>
+          <t>Aug 28</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="13" t="n">
@@ -13658,8 +13697,16 @@
           <t>Blocks sub-study</t>
         </is>
       </c>
-      <c r="E17" s="13" t="n"/>
-      <c r="F17" s="13" t="n"/>
+      <c r="E17" s="13" t="inlineStr">
+        <is>
+          <t>REVISED AND ACCEPTED, confirmed by user 2026-08-28: the rule as originally written only checked memory settings, which can't tell 'platform never read the file' apart from 'platform read it in-conversation but didn't persist it to memory' -- both would look identical (token absent from settings). Added an in-conversation check as an equal, separate passive check alongside the memory-settings check, before the forced-read fallback. Full revised procedure: Upload the file. In the SAME conversation, ask a direct question about the document's content (passive check -- did the platform read the file at all, without being told to summarize?); record whether the token comes back. Separately, check memory/personalization settings for the token (passive check -- did it also get saved to persistent memory?). If the token is absent from BOTH, do a forced-read step (explicitly ask the platform to summarize the document) and recheck both. Log the outcome as one of: extracted into conversation only / extracted into memory only / extracted into both / not extracted until forced / never extracted -- do not collapse into a single 'extraction happened' flag, since in-conversation extraction and persistent-memory extraction are different claims (a platform can read a file fine in-session without ever saving it to long-term memory).</t>
+        </is>
+      </c>
+      <c r="F17" s="13" t="inlineStr">
+        <is>
+          <t>Aug 28</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="13" t="n">

</xml_diff>

<commit_message>
dev::clean up all cells for fresh injection
</commit_message>
<xml_diff>
--- a/RTBF-Prompt/data/RTBF Experiments.xlsx
+++ b/RTBF-Prompt/data/RTBF Experiments.xlsx
@@ -4991,7 +4991,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U89"/>
+  <dimension ref="A1:V89"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="14" customWidth="1" style="22" min="1" max="1"/>
@@ -5122,6 +5122,11 @@
           <t>Disclosure sentence (varied carrier, 2026-08-24)</t>
         </is>
       </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="13" t="inlineStr">
@@ -5166,7 +5171,7 @@
       </c>
       <c r="I2" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J2" s="13" t="n"/>
@@ -5175,7 +5180,11 @@
       <c r="M2" s="13" t="n"/>
       <c r="N2" s="13" t="n"/>
       <c r="O2" s="13" t="n"/>
-      <c r="P2" s="13" t="n"/>
+      <c r="P2" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-08-28T08:53:43.629559+00:00</t>
+        </is>
+      </c>
       <c r="Q2" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -5188,6 +5197,11 @@
           <t>small update: a vegetable patch out back is called "Algorithm Alabaster Muck Borax" as of yesterday</t>
         </is>
       </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
@@ -5232,7 +5246,7 @@
       </c>
       <c r="I3" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J3" s="13" t="n"/>
@@ -5241,7 +5255,11 @@
       <c r="M3" s="13" t="n"/>
       <c r="N3" s="13" t="n"/>
       <c r="O3" s="13" t="n"/>
-      <c r="P3" s="13" t="n"/>
+      <c r="P3" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-08-28T08:53:56.253866+00:00</t>
+        </is>
+      </c>
       <c r="Q3" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -5253,6 +5271,11 @@
           <t>oh random thing -- ended up naming a bonsai tree I'm training "Constable Axis Catching"</t>
         </is>
       </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="13" t="inlineStr">
@@ -5297,7 +5320,7 @@
       </c>
       <c r="I4" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J4" s="13" t="n"/>
@@ -5306,7 +5329,11 @@
       <c r="M4" s="13" t="n"/>
       <c r="N4" s="13" t="n"/>
       <c r="O4" s="13" t="n"/>
-      <c r="P4" s="13" t="n"/>
+      <c r="P4" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-08-28T08:54:14.798306+00:00</t>
+        </is>
+      </c>
       <c r="Q4" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -5318,6 +5345,11 @@
           <t>lol also a compost bin in the backyard is officially "Geranium Sympathy" now</t>
         </is>
       </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="13" t="inlineStr">
@@ -5362,7 +5394,7 @@
       </c>
       <c r="I5" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J5" s="13" t="n"/>
@@ -5371,7 +5403,11 @@
       <c r="M5" s="13" t="n"/>
       <c r="N5" s="13" t="n"/>
       <c r="O5" s="13" t="n"/>
-      <c r="P5" s="13" t="n"/>
+      <c r="P5" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-09-01T07:14:40.309609+00:00</t>
+        </is>
+      </c>
       <c r="Q5" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -5388,6 +5424,11 @@
           <t>side note, went with "Quirk Backspace Bucket" for my old guitar</t>
         </is>
       </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="13" t="inlineStr">
@@ -5432,7 +5473,7 @@
       </c>
       <c r="I6" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J6" s="13" t="n"/>
@@ -5441,7 +5482,11 @@
       <c r="M6" s="13" t="n"/>
       <c r="N6" s="13" t="n"/>
       <c r="O6" s="13" t="n"/>
-      <c r="P6" s="13" t="n"/>
+      <c r="P6" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-08-28T08:54:32.382203+00:00 | auto-injected 2026-09-01T06:24:30.447738+00:00</t>
+        </is>
+      </c>
       <c r="Q6" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -5453,6 +5498,11 @@
           <t>small update: a sketchbook I've been filling is called "Chomp Dynamic Daybreak Overhang" as of yesterday</t>
         </is>
       </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>olabamipet@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="13" t="inlineStr">
@@ -5497,7 +5547,7 @@
       </c>
       <c r="I7" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J7" s="13" t="inlineStr">
@@ -5518,7 +5568,11 @@
       <c r="M7" s="13" t="n"/>
       <c r="N7" s="13" t="n"/>
       <c r="O7" s="13" t="n"/>
-      <c r="P7" s="13" t="n"/>
+      <c r="P7" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-08-28T08:54:50.937169+00:00</t>
+        </is>
+      </c>
       <c r="Q7" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -5530,6 +5584,11 @@
           <t>hey, can you remember this -- a pottery piece I'm working on is named "Doormat Bleach Supremacy Psychic"</t>
         </is>
       </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="13" t="inlineStr">
@@ -5574,7 +5633,7 @@
       </c>
       <c r="I8" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J8" s="13" t="n"/>
@@ -5583,7 +5642,11 @@
       <c r="M8" s="13" t="n"/>
       <c r="N8" s="13" t="n"/>
       <c r="O8" s="13" t="n"/>
-      <c r="P8" s="13" t="n"/>
+      <c r="P8" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-08-28T08:55:07.512750+00:00</t>
+        </is>
+      </c>
       <c r="Q8" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -5595,6 +5658,11 @@
           <t>please make a note that a woodworking project in the garage is called "Provider Refining Breeze"</t>
         </is>
       </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="13" t="inlineStr">
@@ -5639,7 +5707,7 @@
       </c>
       <c r="I9" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J9" s="13" t="n"/>
@@ -5648,7 +5716,11 @@
       <c r="M9" s="13" t="n"/>
       <c r="N9" s="13" t="n"/>
       <c r="O9" s="13" t="n"/>
-      <c r="P9" s="13" t="n"/>
+      <c r="P9" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-08-28T08:55:23.997196+00:00</t>
+        </is>
+      </c>
       <c r="Q9" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -5660,6 +5732,11 @@
           <t>I want you to remember: a quilt I'm sewing = "Starlight Escalator" from now on</t>
         </is>
       </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="13" t="inlineStr">
@@ -5704,7 +5781,7 @@
       </c>
       <c r="I10" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J10" s="13" t="n"/>
@@ -5713,7 +5790,11 @@
       <c r="M10" s="13" t="n"/>
       <c r="N10" s="13" t="n"/>
       <c r="O10" s="13" t="n"/>
-      <c r="P10" s="13" t="n"/>
+      <c r="P10" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-09-01T07:15:01.141610+00:00</t>
+        </is>
+      </c>
       <c r="Q10" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -5730,6 +5811,11 @@
           <t>can you save this for later -- a scarf I'm knitting goes by "Stash Silver Broadside Caption"</t>
         </is>
       </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="13" t="inlineStr">
@@ -5774,7 +5860,7 @@
       </c>
       <c r="I11" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J11" s="13" t="n"/>
@@ -5783,7 +5869,11 @@
       <c r="M11" s="13" t="n"/>
       <c r="N11" s="13" t="n"/>
       <c r="O11" s="13" t="n"/>
-      <c r="P11" s="13" t="n"/>
+      <c r="P11" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-08-28T08:55:41.528334+00:00 | auto-injected 2026-09-01T06:25:06.801389+00:00 | auto-injected 2026-09-01T06:27:27.700845+00:00 | auto-injected 2026-09-01T06:32:53.310499+00:00</t>
+        </is>
+      </c>
       <c r="Q11" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -5795,6 +5885,11 @@
           <t>hey, can you remember this -- a birdhouse I built is named "Action Division"</t>
         </is>
       </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>experimentanchor@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="13" t="inlineStr">
@@ -5839,7 +5934,7 @@
       </c>
       <c r="I12" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J12" s="13" t="inlineStr">
@@ -5860,7 +5955,11 @@
       <c r="M12" s="13" t="n"/>
       <c r="N12" s="13" t="n"/>
       <c r="O12" s="13" t="n"/>
-      <c r="P12" s="13" t="n"/>
+      <c r="P12" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-08-28T08:55:59.810797+00:00</t>
+        </is>
+      </c>
       <c r="Q12" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -5872,6 +5971,11 @@
           <t>FYI -- a terrarium I put together is called "Crispness Dove Showdown Backing".</t>
         </is>
       </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="13" t="inlineStr">
@@ -5916,7 +6020,7 @@
       </c>
       <c r="I13" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J13" s="13" t="n"/>
@@ -5925,7 +6029,11 @@
       <c r="M13" s="13" t="n"/>
       <c r="N13" s="13" t="n"/>
       <c r="O13" s="13" t="n"/>
-      <c r="P13" s="13" t="n"/>
+      <c r="P13" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-08-28T08:56:17.610743+00:00</t>
+        </is>
+      </c>
       <c r="Q13" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -5937,6 +6045,11 @@
           <t>FYI -- a scrapbook I'm making is called "Earlobe Parlor".</t>
         </is>
       </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="13" t="inlineStr">
@@ -5981,7 +6094,7 @@
       </c>
       <c r="I14" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J14" s="13" t="n"/>
@@ -5990,7 +6103,11 @@
       <c r="M14" s="13" t="n"/>
       <c r="N14" s="13" t="n"/>
       <c r="O14" s="13" t="n"/>
-      <c r="P14" s="13" t="n"/>
+      <c r="P14" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-08-28T08:56:35.456265+00:00</t>
+        </is>
+      </c>
       <c r="Q14" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -6002,6 +6119,11 @@
           <t>FYI -- a jigsaw puzzle on the coffee table is called "Barterer Earflap Washhouse".</t>
         </is>
       </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="13" t="inlineStr">
@@ -6046,7 +6168,7 @@
       </c>
       <c r="I15" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J15" s="13" t="n"/>
@@ -6055,7 +6177,11 @@
       <c r="M15" s="13" t="n"/>
       <c r="N15" s="13" t="n"/>
       <c r="O15" s="13" t="n"/>
-      <c r="P15" s="13" t="n"/>
+      <c r="P15" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-09-01T07:15:43.096114+00:00</t>
+        </is>
+      </c>
       <c r="Q15" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -6072,6 +6198,11 @@
           <t>FYI -- a chess set I got as a gift is called "Debit Bulb Ankle".</t>
         </is>
       </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="13" t="inlineStr">
@@ -6116,7 +6247,7 @@
       </c>
       <c r="I16" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J16" s="13" t="n"/>
@@ -6125,7 +6256,11 @@
       <c r="M16" s="13" t="n"/>
       <c r="N16" s="13" t="n"/>
       <c r="O16" s="13" t="n"/>
-      <c r="P16" s="13" t="n"/>
+      <c r="P16" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-08-28T08:56:53.488007+00:00 | auto-injected 2026-09-01T06:46:28.093785+00:00</t>
+        </is>
+      </c>
       <c r="Q16" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -6135,6 +6270,11 @@
       <c r="U16" s="0" t="inlineStr">
         <is>
           <t>FYI -- a photo album I'm putting together is called "Gift Amends".</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>olacoderpad@gmail.com</t>
         </is>
       </c>
     </row>
@@ -6241,7 +6381,7 @@
       </c>
       <c r="I20" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J20" s="13" t="n"/>
@@ -6250,7 +6390,11 @@
       <c r="M20" s="13" t="n"/>
       <c r="N20" s="13" t="n"/>
       <c r="O20" s="13" t="n"/>
-      <c r="P20" s="13" t="n"/>
+      <c r="P20" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-09-01T07:20:41.805949+00:00</t>
+        </is>
+      </c>
       <c r="Q20" s="13" t="inlineStr">
         <is>
           <t>Expected FAIL same-session: dry run showed NL forget leaves data recallable while model confirms deletion.</t>
@@ -6269,6 +6413,11 @@
       <c r="U20" s="0" t="inlineStr">
         <is>
           <t>oh random thing -- ended up naming a new houseplant "Ninth Barge Renovator"</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>olacoderpad@gmail.com</t>
         </is>
       </c>
     </row>
@@ -6315,7 +6464,7 @@
       </c>
       <c r="I21" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>ERASED</t>
         </is>
       </c>
       <c r="J21" s="13" t="n"/>
@@ -6324,7 +6473,11 @@
       <c r="M21" s="13" t="n"/>
       <c r="N21" s="13" t="n"/>
       <c r="O21" s="13" t="n"/>
-      <c r="P21" s="13" t="n"/>
+      <c r="P21" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-08-28T08:57:08.834302+00:00 | auto-erased 2026-08-31T05:28:01.873386+00:00</t>
+        </is>
+      </c>
       <c r="Q21" s="13" t="inlineStr">
         <is>
           <t>Expected FAIL (anchor survives): dry run showed conversation deletion is UI-only (is_visible:false); memory-extracted content persists.</t>
@@ -6338,6 +6491,11 @@
       <c r="U21" s="0" t="inlineStr">
         <is>
           <t>lol also my sourdough starter culture is officially "Skinny Stopper" now</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>olacoderpad@gmail.com</t>
         </is>
       </c>
     </row>
@@ -6384,7 +6542,7 @@
       </c>
       <c r="I22" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J22" s="13" t="n"/>
@@ -6393,7 +6551,11 @@
       <c r="M22" s="13" t="n"/>
       <c r="N22" s="13" t="n"/>
       <c r="O22" s="13" t="n"/>
-      <c r="P22" s="13" t="n"/>
+      <c r="P22" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-08-28T08:57:25.216866+00:00</t>
+        </is>
+      </c>
       <c r="Q22" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -6405,6 +6567,11 @@
           <t>small update: a side project I'm tinkering with is called "Galleria Camper Nemeses" as of yesterday</t>
         </is>
       </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>olacoderpad@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="13" t="inlineStr">
@@ -6449,7 +6616,7 @@
       </c>
       <c r="I23" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>ERASED</t>
         </is>
       </c>
       <c r="J23" s="13" t="n"/>
@@ -6460,7 +6627,7 @@
       <c r="O23" s="13" t="n"/>
       <c r="P23" s="13" t="inlineStr">
         <is>
-          <t>Confirmed live 2026-08-27: genuine text field with an explicit Save button (does not autosave on blur) -- resolves Q6, no toggle-vs-field ambiguity.</t>
+          <t>Confirmed live 2026-08-27: genuine text field with an explicit Save button (does not autosave on blur) -- resolves Q6, no toggle-vs-field ambiguity. | auto-injected 2026-08-28T08:57:39.796004+00:00 | auto-erased 2026-08-31T05:28:32.702299+00:00</t>
         </is>
       </c>
       <c r="Q23" s="13" t="inlineStr">
@@ -6474,6 +6641,11 @@
           <t>oh random thing -- ended up naming a playlist I made "Skipper Splendor Feminine"</t>
         </is>
       </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>olacoderpad@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="15.75" customHeight="1" s="22">
       <c r="A24" s="13" t="inlineStr">
@@ -6518,7 +6690,7 @@
       </c>
       <c r="I24" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J24" s="13" t="n"/>
@@ -6527,7 +6699,11 @@
       <c r="M24" s="13" t="n"/>
       <c r="N24" s="13" t="n"/>
       <c r="O24" s="13" t="n"/>
-      <c r="P24" s="13" t="n"/>
+      <c r="P24" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-08-28T08:57:54.599232+00:00</t>
+        </is>
+      </c>
       <c r="Q24" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -6539,6 +6715,11 @@
           <t>lol also our home renovation is officially "Justifier Security Haunt Tightness" now</t>
         </is>
       </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>olacoderpad@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="15.75" customHeight="1" s="22">
       <c r="A25" s="13" t="inlineStr">
@@ -6583,7 +6764,7 @@
       </c>
       <c r="I25" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J25" s="13" t="n"/>
@@ -6592,7 +6773,11 @@
       <c r="M25" s="13" t="n"/>
       <c r="N25" s="13" t="n"/>
       <c r="O25" s="13" t="n"/>
-      <c r="P25" s="13" t="n"/>
+      <c r="P25" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-08-28T08:58:12.958010+00:00 | auto-injected 2026-09-01T04:57:33.708144+00:00</t>
+        </is>
+      </c>
       <c r="Q25" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -6604,6 +6789,11 @@
           <t>side note, went with "Ranking Wisdom" for the garden bed I just planted</t>
         </is>
       </c>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>olabamipet@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="15.75" customHeight="1" s="22">
       <c r="A26" s="13" t="inlineStr">
@@ -6648,7 +6838,7 @@
       </c>
       <c r="I26" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J26" s="13" t="n"/>
@@ -6657,7 +6847,11 @@
       <c r="M26" s="13" t="n"/>
       <c r="N26" s="13" t="n"/>
       <c r="O26" s="13" t="n"/>
-      <c r="P26" s="13" t="n"/>
+      <c r="P26" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-09-01T07:20:59.758460+00:00</t>
+        </is>
+      </c>
       <c r="Q26" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -6674,6 +6868,11 @@
           <t>can you save this for later -- a new bike goes by "Spinner Follicle"</t>
         </is>
       </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>olacoderpad@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="15.75" customHeight="1" s="22">
       <c r="A27" s="13" t="inlineStr">
@@ -6718,7 +6917,7 @@
       </c>
       <c r="I27" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>ERASED</t>
         </is>
       </c>
       <c r="J27" s="13" t="n"/>
@@ -6727,7 +6926,11 @@
       <c r="M27" s="13" t="n"/>
       <c r="N27" s="13" t="n"/>
       <c r="O27" s="13" t="n"/>
-      <c r="P27" s="13" t="n"/>
+      <c r="P27" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-08-28T08:58:26.624789+00:00 | auto-erased 2026-08-31T05:28:09.859564+00:00</t>
+        </is>
+      </c>
       <c r="Q27" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -6739,6 +6942,11 @@
           <t>hey, can you remember this -- my old car is named "Nutcase Taps"</t>
         </is>
       </c>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>olacoderpad@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="15.75" customHeight="1" s="22">
       <c r="A28" s="13" t="inlineStr">
@@ -6783,7 +6991,7 @@
       </c>
       <c r="I28" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J28" s="13" t="n"/>
@@ -6792,7 +7000,11 @@
       <c r="M28" s="13" t="n"/>
       <c r="N28" s="13" t="n"/>
       <c r="O28" s="13" t="n"/>
-      <c r="P28" s="13" t="n"/>
+      <c r="P28" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-08-28T08:58:41.053858+00:00</t>
+        </is>
+      </c>
       <c r="Q28" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -6804,6 +7016,11 @@
           <t>I want you to remember: a motorcycle I'm fixing up = "Jaundice Supper Gauntlet" from now on</t>
         </is>
       </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>olacoderpad@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="15.75" customHeight="1" s="22">
       <c r="A29" s="13" t="inlineStr">
@@ -6848,7 +7065,7 @@
       </c>
       <c r="I29" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J29" s="13" t="n"/>
@@ -6859,7 +7076,7 @@
       <c r="O29" s="13" t="n"/>
       <c r="P29" s="13" t="inlineStr">
         <is>
-          <t>Confirmed live 2026-08-27: genuine text field with an explicit Save button (does not autosave on blur) -- resolves Q6, no toggle-vs-field ambiguity.</t>
+          <t>Confirmed live 2026-08-27: genuine text field with an explicit Save button (does not autosave on blur) -- resolves Q6, no toggle-vs-field ambiguity. | auto-injected 2026-08-28T08:58:55.273241+00:00</t>
         </is>
       </c>
       <c r="Q29" s="13" t="inlineStr">
@@ -6873,6 +7090,11 @@
           <t>can you save this for later -- a canoe we restored goes by "Wrist Endpoint Denim"</t>
         </is>
       </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>olacoderpad@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="15.75" customHeight="1" s="22">
       <c r="A30" s="13" t="inlineStr">
@@ -6917,7 +7139,7 @@
       </c>
       <c r="I30" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J30" s="13" t="n"/>
@@ -6926,7 +7148,11 @@
       <c r="M30" s="13" t="n"/>
       <c r="N30" s="13" t="n"/>
       <c r="O30" s="13" t="n"/>
-      <c r="P30" s="13" t="n"/>
+      <c r="P30" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-08-28T08:59:09.539180+00:00</t>
+        </is>
+      </c>
       <c r="Q30" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -6938,6 +7164,11 @@
           <t>hey, can you remember this -- an electric scooter I got is named "Abacus Engine Backside Kilobyte"</t>
         </is>
       </c>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>olacoderpad@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="15.75" customHeight="1" s="22">
       <c r="A31" s="13" t="inlineStr">
@@ -6982,7 +7213,7 @@
       </c>
       <c r="I31" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J31" s="13" t="n"/>
@@ -6991,7 +7222,11 @@
       <c r="M31" s="13" t="n"/>
       <c r="N31" s="13" t="n"/>
       <c r="O31" s="13" t="n"/>
-      <c r="P31" s="13" t="n"/>
+      <c r="P31" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-08-28T08:59:23.791561+00:00 | auto-injected 2026-09-01T06:52:16.636505+00:00</t>
+        </is>
+      </c>
       <c r="Q31" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -7003,6 +7238,11 @@
           <t>please make a note that a puppy we just adopted is called "Cheating Mauve"</t>
         </is>
       </c>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>experimentanchor@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="15.75" customHeight="1" s="22">
       <c r="A32" s="13" t="inlineStr">
@@ -7047,7 +7287,7 @@
       </c>
       <c r="I32" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J32" s="13" t="n"/>
@@ -7056,7 +7296,11 @@
       <c r="M32" s="13" t="n"/>
       <c r="N32" s="13" t="n"/>
       <c r="O32" s="13" t="n"/>
-      <c r="P32" s="13" t="n"/>
+      <c r="P32" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-09-01T07:21:14.731576+00:00</t>
+        </is>
+      </c>
       <c r="Q32" s="13" t="inlineStr">
         <is>
           <t>EXPECTED-NULL: NL forget does not modify custom instructions field.</t>
@@ -7075,6 +7319,11 @@
       <c r="U32" s="0" t="inlineStr">
         <is>
           <t>FYI -- a kitten we're fostering is called "Stability Problem Hydroxide Compare".</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>olacoderpad@gmail.com</t>
         </is>
       </c>
     </row>
@@ -7121,7 +7370,7 @@
       </c>
       <c r="I33" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J33" s="13" t="n"/>
@@ -7130,7 +7379,11 @@
       <c r="M33" s="13" t="n"/>
       <c r="N33" s="13" t="n"/>
       <c r="O33" s="13" t="n"/>
-      <c r="P33" s="13" t="n"/>
+      <c r="P33" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-08-28T08:59:34.034111+00:00 | auto-erased 2026-08-31T05:28:17.637620+00:00 | auto-injected 2026-08-31T06:11:10.959928+00:00</t>
+        </is>
+      </c>
       <c r="Q33" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -7142,6 +7395,11 @@
           <t>FYI -- a rescue dog we brought home is called "Importer Carat Valuables Marathon".</t>
         </is>
       </c>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>olacoderpad@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="15.75" customHeight="1" s="22">
       <c r="A34" s="13" t="inlineStr">
@@ -7186,7 +7444,7 @@
       </c>
       <c r="I34" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J34" s="13" t="n"/>
@@ -7195,7 +7453,11 @@
       <c r="M34" s="13" t="n"/>
       <c r="N34" s="13" t="n"/>
       <c r="O34" s="13" t="n"/>
-      <c r="P34" s="13" t="n"/>
+      <c r="P34" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-08-28T08:59:44.014026+00:00 | auto-injected 2026-08-31T06:11:23.705916+00:00</t>
+        </is>
+      </c>
       <c r="Q34" s="13" t="inlineStr">
         <is>
           <t>EXPECTED-NULL: clear-all memories does not reach custom instructions.</t>
@@ -7209,6 +7471,11 @@
       <c r="U34" s="0" t="inlineStr">
         <is>
           <t>FYI -- a hamster the kids got is called "Snack Shame".</t>
+        </is>
+      </c>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>olacoderpad@gmail.com</t>
         </is>
       </c>
     </row>
@@ -7255,7 +7522,7 @@
       </c>
       <c r="I35" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J35" s="13" t="n"/>
@@ -7266,7 +7533,7 @@
       <c r="O35" s="13" t="n"/>
       <c r="P35" s="13" t="inlineStr">
         <is>
-          <t>Confirmed live 2026-08-27: genuine text field with an explicit Save button (does not autosave on blur) -- resolves Q6, no toggle-vs-field ambiguity.</t>
+          <t>Confirmed live 2026-08-27: genuine text field with an explicit Save button (does not autosave on blur) -- resolves Q6, no toggle-vs-field ambiguity. | auto-injected 2026-08-28T08:59:54.331966+00:00 | auto-injected 2026-08-31T06:11:35.662279+00:00</t>
         </is>
       </c>
       <c r="Q35" s="13" t="inlineStr">
@@ -7280,6 +7547,11 @@
           <t>FYI -- a backyard chicken coop is called "Driver Taunt Ribbon".</t>
         </is>
       </c>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>olacoderpad@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="15.75" customHeight="1" s="22">
       <c r="A36" s="13" t="inlineStr">
@@ -7324,7 +7596,7 @@
       </c>
       <c r="I36" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J36" s="13" t="n"/>
@@ -7333,7 +7605,11 @@
       <c r="M36" s="13" t="n"/>
       <c r="N36" s="13" t="n"/>
       <c r="O36" s="13" t="n"/>
-      <c r="P36" s="13" t="n"/>
+      <c r="P36" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-08-28T09:00:04.639086+00:00 | auto-injected 2026-08-31T06:11:48.023112+00:00</t>
+        </is>
+      </c>
       <c r="Q36" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -7345,6 +7621,11 @@
           <t>FYI -- a tomato plant on the balcony is called "Tuition Barge".</t>
         </is>
       </c>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>olacoderpad@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="15.75" customHeight="1" s="22">
       <c r="A37" s="13" t="inlineStr">
@@ -7389,7 +7670,7 @@
       </c>
       <c r="I37" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J37" s="13" t="n"/>
@@ -7398,7 +7679,11 @@
       <c r="M37" s="13" t="n"/>
       <c r="N37" s="13" t="n"/>
       <c r="O37" s="13" t="n"/>
-      <c r="P37" s="13" t="n"/>
+      <c r="P37" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-08-28T09:00:14.850606+00:00 | auto-injected 2026-09-01T06:52:48.819159+00:00</t>
+        </is>
+      </c>
       <c r="Q37" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -7408,6 +7693,11 @@
       <c r="U37" s="0" t="inlineStr">
         <is>
           <t>FYI -- an herb garden I started is called "Graph Ranting".</t>
+        </is>
+      </c>
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>anchorexperiment+001@gmail.com</t>
         </is>
       </c>
     </row>
@@ -7514,7 +7804,7 @@
       </c>
       <c r="I41" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J41" s="13" t="n"/>
@@ -7523,7 +7813,11 @@
       <c r="M41" s="13" t="n"/>
       <c r="N41" s="13" t="n"/>
       <c r="O41" s="13" t="n"/>
-      <c r="P41" s="13" t="n"/>
+      <c r="P41" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-09-01T07:21:51.710790+00:00</t>
+        </is>
+      </c>
       <c r="Q41" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -7540,6 +7834,11 @@
           <t>oh random thing -- ended up naming a language app streak I'm keeping up "Walrus Scooter Hunchback Subject"</t>
         </is>
       </c>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="15.75" customHeight="1" s="22">
       <c r="A42" s="13" t="inlineStr">
@@ -7584,7 +7883,7 @@
       </c>
       <c r="I42" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J42" s="13" t="n"/>
@@ -7593,7 +7892,11 @@
       <c r="M42" s="13" t="n"/>
       <c r="N42" s="13" t="n"/>
       <c r="O42" s="13" t="n"/>
-      <c r="P42" s="13" t="n"/>
+      <c r="P42" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-08-28T09:00:30.982335+00:00</t>
+        </is>
+      </c>
       <c r="Q42" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -7605,6 +7908,11 @@
           <t>lol also our vacation itinerary is officially "Lavender Juggling" now</t>
         </is>
       </c>
+      <c r="V42" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="15.75" customHeight="1" s="22">
       <c r="A43" s="13" t="inlineStr">
@@ -7649,7 +7957,7 @@
       </c>
       <c r="I43" s="13" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J43" s="13" t="n"/>
@@ -7660,7 +7968,7 @@
       <c r="O43" s="13" t="n"/>
       <c r="P43" s="13" t="inlineStr">
         <is>
-          <t>CONFIRMED DEAD END (2026-08-28): 5 independent live attempts, all failed identically -- cookie replay (stale + fresh, tested within 1 min of export), in-app click-through, playwright-stealth, and an alternate in-product path (dead end, links to a help article). Matches this project's documented pattern of Google rejecting any CDP-driven browser regardless of cookie validity (see ChatGPT OAuth finding). Run by hand. See DECISIONS Q20 and flows/gemini.py's _delete_all_activity() docstring for the full investigation.</t>
+          <t>CONFIRMED DEAD END (2026-08-28): 5 independent live attempts, all failed identically -- cookie replay (stale + fresh, tested within 1 min of export), in-app click-through, playwright-stealth, and an alternate in-product path (dead end, links to a help article). Matches this project's documented pattern of Google rejecting any CDP-driven browser regardless of cookie validity (see ChatGPT OAuth finding). Run by hand. See DECISIONS Q20 and flows/gemini.py's _delete_all_activity() docstring for the full investigation. | auto-injected 2026-08-28T09:00:44.049128+00:00</t>
         </is>
       </c>
       <c r="Q43" s="13" t="inlineStr">
@@ -7674,6 +7982,11 @@
           <t>side note, went with "Breach Opacity" for a camping trip I'm organizing</t>
         </is>
       </c>
+      <c r="V43" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="15.75" customHeight="1" s="22">
       <c r="A44" s="13" t="inlineStr">
@@ -7718,7 +8031,7 @@
       </c>
       <c r="I44" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J44" s="13" t="n"/>
@@ -7727,7 +8040,11 @@
       <c r="M44" s="13" t="n"/>
       <c r="N44" s="13" t="n"/>
       <c r="O44" s="13" t="n"/>
-      <c r="P44" s="13" t="n"/>
+      <c r="P44" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-08-28T09:10:48.234542+00:00</t>
+        </is>
+      </c>
       <c r="Q44" s="13" t="inlineStr">
         <is>
           <t>EXPECTED-NULL: anchor survives. Saved-info deletion does not reach conversational layer; conversational data does not enter Saved info.</t>
@@ -7741,6 +8058,11 @@
       <c r="U44" s="0" t="inlineStr">
         <is>
           <t>small update: a hiking trail I want to do is called "Landfall Finisher Silencer Sash" as of yesterday</t>
+        </is>
+      </c>
+      <c r="V44" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
         </is>
       </c>
     </row>
@@ -7787,7 +8109,7 @@
       </c>
       <c r="I45" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J45" s="13" t="n"/>
@@ -7796,7 +8118,11 @@
       <c r="M45" s="13" t="n"/>
       <c r="N45" s="13" t="n"/>
       <c r="O45" s="13" t="n"/>
-      <c r="P45" s="13" t="n"/>
+      <c r="P45" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-08-28T09:02:07.936597+00:00</t>
+        </is>
+      </c>
       <c r="Q45" s="13" t="inlineStr">
         <is>
           <t>EXPECTED-NULL: anchor survives. Same scope limit as E4.</t>
@@ -7810,6 +8136,11 @@
       <c r="U45" s="0" t="inlineStr">
         <is>
           <t>oh random thing -- ended up naming a weekend getaway I'm planning "Refueling Navigator Mutation"</t>
+        </is>
+      </c>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
         </is>
       </c>
     </row>
@@ -7856,7 +8187,7 @@
       </c>
       <c r="I46" s="13" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J46" s="13" t="n"/>
@@ -7867,7 +8198,7 @@
       <c r="O46" s="13" t="n"/>
       <c r="P46" s="13" t="inlineStr">
         <is>
-          <t>CONFIRMED DEAD END (2026-08-28): 5 independent live attempts, all failed identically -- cookie replay (stale + fresh, tested within 1 min of export), in-app click-through, playwright-stealth, and an alternate in-product path (dead end, links to a help article). Matches this project's documented pattern of Google rejecting any CDP-driven browser regardless of cookie validity (see ChatGPT OAuth finding). Run by hand. See DECISIONS Q20 and flows/gemini.py's _delete_all_activity() docstring for the full investigation.</t>
+          <t>CONFIRMED DEAD END (2026-08-28): 5 independent live attempts, all failed identically -- cookie replay (stale + fresh, tested within 1 min of export), in-app click-through, playwright-stealth, and an alternate in-product path (dead end, links to a help article). Matches this project's documented pattern of Google rejecting any CDP-driven browser regardless of cookie validity (see ChatGPT OAuth finding). Run by hand. See DECISIONS Q20 and flows/gemini.py's _delete_all_activity() docstring for the full investigation. | auto-injected 2026-08-28T09:02:21.633981+00:00 | auto-injected 2026-09-01T06:54:27.486439+00:00</t>
         </is>
       </c>
       <c r="Q46" s="13" t="inlineStr">
@@ -7881,6 +8212,11 @@
           <t>lol also my vinyl record collection is officially "Skeptic Earful" now</t>
         </is>
       </c>
+      <c r="V46" t="inlineStr">
+        <is>
+          <t>olabamipet@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="15.75" customHeight="1" s="22">
       <c r="A47" s="13" t="inlineStr">
@@ -7925,7 +8261,7 @@
       </c>
       <c r="I47" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J47" s="13" t="n"/>
@@ -7934,7 +8270,11 @@
       <c r="M47" s="13" t="n"/>
       <c r="N47" s="13" t="n"/>
       <c r="O47" s="13" t="n"/>
-      <c r="P47" s="13" t="n"/>
+      <c r="P47" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-09-01T07:24:32.717087+00:00</t>
+        </is>
+      </c>
       <c r="Q47" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -7951,6 +8291,11 @@
           <t>I want you to remember: a stamp collection I inherited = "Juggle Imagines" from now on</t>
         </is>
       </c>
+      <c r="V47" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="15.75" customHeight="1" s="22">
       <c r="A48" s="13" t="inlineStr">
@@ -7995,7 +8340,7 @@
       </c>
       <c r="I48" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J48" s="13" t="n"/>
@@ -8004,7 +8349,11 @@
       <c r="M48" s="13" t="n"/>
       <c r="N48" s="13" t="n"/>
       <c r="O48" s="13" t="n"/>
-      <c r="P48" s="13" t="n"/>
+      <c r="P48" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-08-28T09:02:37.221770+00:00</t>
+        </is>
+      </c>
       <c r="Q48" s="13" t="inlineStr">
         <is>
           <t>EXPECTED-NULL: anchor survives. Conversation deletion does not reach Saved info layer.</t>
@@ -8018,6 +8367,11 @@
       <c r="U48" s="0" t="inlineStr">
         <is>
           <t>can you save this for later -- a rock and mineral collection goes by "Aching Uplifting Theater"</t>
+        </is>
+      </c>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
         </is>
       </c>
     </row>
@@ -8064,7 +8418,7 @@
       </c>
       <c r="I49" s="13" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J49" s="13" t="n"/>
@@ -8075,7 +8429,7 @@
       <c r="O49" s="13" t="n"/>
       <c r="P49" s="13" t="inlineStr">
         <is>
-          <t>CONFIRMED DEAD END (2026-08-28): 5 independent live attempts, all failed identically -- cookie replay (stale + fresh, tested within 1 min of export), in-app click-through, playwright-stealth, and an alternate in-product path (dead end, links to a help article). Matches this project's documented pattern of Google rejecting any CDP-driven browser regardless of cookie validity (see ChatGPT OAuth finding). Run by hand. See DECISIONS Q20 and flows/gemini.py's _delete_all_activity() docstring for the full investigation.</t>
+          <t>CONFIRMED DEAD END (2026-08-28): 5 independent live attempts, all failed identically -- cookie replay (stale + fresh, tested within 1 min of export), in-app click-through, playwright-stealth, and an alternate in-product path (dead end, links to a help article). Matches this project's documented pattern of Google rejecting any CDP-driven browser regardless of cookie validity (see ChatGPT OAuth finding). Run by hand. See DECISIONS Q20 and flows/gemini.py's _delete_all_activity() docstring for the full investigation. | auto-injected 2026-08-28T09:02:52.446711+00:00</t>
         </is>
       </c>
       <c r="Q49" s="13" t="inlineStr">
@@ -8089,6 +8443,11 @@
           <t>hey, can you remember this -- a comic book collection is named "Antonym August Dude Shadow"</t>
         </is>
       </c>
+      <c r="V49" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="15.75" customHeight="1" s="22">
       <c r="A50" s="13" t="inlineStr">
@@ -8133,7 +8492,7 @@
       </c>
       <c r="I50" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J50" s="13" t="n"/>
@@ -8142,7 +8501,11 @@
       <c r="M50" s="13" t="n"/>
       <c r="N50" s="13" t="n"/>
       <c r="O50" s="13" t="n"/>
-      <c r="P50" s="13" t="n"/>
+      <c r="P50" s="13" t="inlineStr">
+        <is>
+          <t>Disclosure sentence reworded 2026-08-28: original phrasing ("please make a note that ... is called ...") was rejected live by Gemini's Saved-info content validator as not reading like a genuine personal fact. Same token/referent kept, swapped to the "hey, can you remember this -- X is named Y" carrier template (already confirmed working on GE-I2-E3 with this exact wording). | auto-injected 2026-08-28T09:11:04.755366+00:00</t>
+        </is>
+      </c>
       <c r="Q50" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -8151,7 +8514,12 @@
       <c r="R50" s="13" t="n"/>
       <c r="U50" s="0" t="inlineStr">
         <is>
-          <t>please make a note that a vintage postcard collection is called "Stadium Trance Osmosis Taps"</t>
+          <t>hey, can you remember this -- a vintage postcard collection is named "Stadium Trance Osmosis Taps"</t>
+        </is>
+      </c>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
         </is>
       </c>
     </row>
@@ -8198,7 +8566,7 @@
       </c>
       <c r="I51" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J51" s="13" t="n"/>
@@ -8207,7 +8575,11 @@
       <c r="M51" s="13" t="n"/>
       <c r="N51" s="13" t="n"/>
       <c r="O51" s="13" t="n"/>
-      <c r="P51" s="13" t="n"/>
+      <c r="P51" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-08-28T09:03:26.250818+00:00</t>
+        </is>
+      </c>
       <c r="Q51" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -8219,6 +8591,11 @@
           <t>I want you to remember: a houseplant collection = "Dash Muck City Return" from now on</t>
         </is>
       </c>
+      <c r="V51" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="15.75" customHeight="1" s="22">
       <c r="A52" s="13" t="inlineStr">
@@ -8263,7 +8640,7 @@
       </c>
       <c r="I52" s="13" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J52" s="13" t="n"/>
@@ -8274,7 +8651,7 @@
       <c r="O52" s="13" t="n"/>
       <c r="P52" s="13" t="inlineStr">
         <is>
-          <t>CONFIRMED DEAD END (2026-08-28): 5 independent live attempts, all failed identically -- cookie replay (stale + fresh, tested within 1 min of export), in-app click-through, playwright-stealth, and an alternate in-product path (dead end, links to a help article). Matches this project's documented pattern of Google rejecting any CDP-driven browser regardless of cookie validity (see ChatGPT OAuth finding). Run by hand. See DECISIONS Q20 and flows/gemini.py's _delete_all_activity() docstring for the full investigation.</t>
+          <t>CONFIRMED DEAD END (2026-08-28): 5 independent live attempts, all failed identically -- cookie replay (stale + fresh, tested within 1 min of export), in-app click-through, playwright-stealth, and an alternate in-product path (dead end, links to a help article). Matches this project's documented pattern of Google rejecting any CDP-driven browser regardless of cookie validity (see ChatGPT OAuth finding). Run by hand. See DECISIONS Q20 and flows/gemini.py's _delete_all_activity() docstring for the full investigation. | auto-injected 2026-08-28T09:03:42.374831+00:00 | auto-injected 2026-09-01T07:00:52.550677+00:00</t>
         </is>
       </c>
       <c r="Q52" s="13" t="inlineStr">
@@ -8286,6 +8663,11 @@
       <c r="U52" s="0" t="inlineStr">
         <is>
           <t>can you save this for later -- a sneaker collection goes by "Marshland Bovine"</t>
+        </is>
+      </c>
+      <c r="V52" t="inlineStr">
+        <is>
+          <t>olacoderpad@gmail.com</t>
         </is>
       </c>
     </row>
@@ -8392,7 +8774,7 @@
       </c>
       <c r="I56" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J56" s="13" t="n"/>
@@ -8401,7 +8783,11 @@
       <c r="M56" s="13" t="n"/>
       <c r="N56" s="13" t="n"/>
       <c r="O56" s="13" t="n"/>
-      <c r="P56" s="13" t="n"/>
+      <c r="P56" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-08-28T09:04:02.626721+00:00</t>
+        </is>
+      </c>
       <c r="Q56" s="13" t="inlineStr">
         <is>
           <t>Expected PASS cross-session (dry run: effective both surfaces); same-session unresolved.</t>
@@ -8415,6 +8801,11 @@
       <c r="U56" s="0" t="inlineStr">
         <is>
           <t>oh random thing -- ended up naming a mural I'm painting in the hallway "Clover Judiciary Blemish"</t>
+        </is>
+      </c>
+      <c r="V56" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
         </is>
       </c>
     </row>
@@ -8461,7 +8852,7 @@
       </c>
       <c r="I57" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J57" s="13" t="n"/>
@@ -8470,7 +8861,11 @@
       <c r="M57" s="13" t="n"/>
       <c r="N57" s="13" t="n"/>
       <c r="O57" s="13" t="n"/>
-      <c r="P57" s="13" t="n"/>
+      <c r="P57" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-08-28T09:04:20.182417+00:00</t>
+        </is>
+      </c>
       <c r="Q57" s="13" t="inlineStr">
         <is>
           <t>Expected FAIL: dry run showed memory deletion leaves conversation history intact; full recall.</t>
@@ -8484,6 +8879,11 @@
       <c r="U57" s="0" t="inlineStr">
         <is>
           <t>lol also a treehouse project for the kids is officially "Vaporizer Pretext Subscript Clip" now</t>
+        </is>
+      </c>
+      <c r="V57" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
         </is>
       </c>
     </row>
@@ -8530,7 +8930,7 @@
       </c>
       <c r="I58" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J58" s="13" t="n"/>
@@ -8539,7 +8939,11 @@
       <c r="M58" s="13" t="n"/>
       <c r="N58" s="13" t="n"/>
       <c r="O58" s="13" t="n"/>
-      <c r="P58" s="13" t="n"/>
+      <c r="P58" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-09-01T07:24:57.002737+00:00</t>
+        </is>
+      </c>
       <c r="Q58" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -8556,6 +8960,11 @@
           <t>side note, went with "Aide Provider Brick Scrounger" for our front yard landscaping</t>
         </is>
       </c>
+      <c r="V58" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="15.75" customHeight="1" s="22">
       <c r="A59" s="13" t="inlineStr">
@@ -8600,7 +9009,7 @@
       </c>
       <c r="I59" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J59" s="13" t="n"/>
@@ -8609,7 +9018,11 @@
       <c r="M59" s="13" t="n"/>
       <c r="N59" s="13" t="n"/>
       <c r="O59" s="13" t="n"/>
-      <c r="P59" s="13" t="n"/>
+      <c r="P59" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-08-28T09:04:36.509077+00:00</t>
+        </is>
+      </c>
       <c r="Q59" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -8621,6 +9034,11 @@
           <t>small update: a fence we're putting up is called "Tabloid Headband" as of yesterday</t>
         </is>
       </c>
+      <c r="V59" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="15.75" customHeight="1" s="22">
       <c r="A60" s="13" t="inlineStr">
@@ -8665,7 +9083,7 @@
       </c>
       <c r="I60" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J60" s="13" t="n"/>
@@ -8674,7 +9092,11 @@
       <c r="M60" s="13" t="n"/>
       <c r="N60" s="13" t="n"/>
       <c r="O60" s="13" t="n"/>
-      <c r="P60" s="13" t="n"/>
+      <c r="P60" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-08-28T09:04:53.111466+00:00</t>
+        </is>
+      </c>
       <c r="Q60" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -8686,6 +9108,11 @@
           <t>oh random thing -- ended up naming a garage workshop I'm setting up "Sternum Sinner Vocalist"</t>
         </is>
       </c>
+      <c r="V60" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="15.75" customHeight="1" s="22">
       <c r="A61" s="13" t="inlineStr">
@@ -8730,7 +9157,7 @@
       </c>
       <c r="I61" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J61" s="13" t="n"/>
@@ -8739,7 +9166,11 @@
       <c r="M61" s="13" t="n"/>
       <c r="N61" s="13" t="n"/>
       <c r="O61" s="13" t="n"/>
-      <c r="P61" s="13" t="n"/>
+      <c r="P61" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-08-28T09:05:09.536688+00:00 | auto-injected 2026-09-01T07:06:25.298557+00:00</t>
+        </is>
+      </c>
       <c r="Q61" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -8751,6 +9182,11 @@
           <t>lol also a mudroom we're adding is officially "Backspin Proponent Scouts Chemicals" now</t>
         </is>
       </c>
+      <c r="V61" t="inlineStr">
+        <is>
+          <t>olabamipet@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="15.75" customHeight="1" s="22">
       <c r="A62" s="13" t="inlineStr">
@@ -8795,7 +9231,7 @@
       </c>
       <c r="I62" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J62" s="13" t="n"/>
@@ -8804,7 +9240,11 @@
       <c r="M62" s="13" t="n"/>
       <c r="N62" s="13" t="n"/>
       <c r="O62" s="13" t="n"/>
-      <c r="P62" s="13" t="n"/>
+      <c r="P62" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-08-28T09:05:25.583715+00:00</t>
+        </is>
+      </c>
       <c r="Q62" s="13" t="inlineStr">
         <is>
           <t>EXPECTED-NULL: conversation deletion does not reach explicit memory store.</t>
@@ -8818,6 +9258,11 @@
       <c r="U62" s="0" t="inlineStr">
         <is>
           <t>I want you to remember: a backyard fire pit we built = "Sandstone Smolder Triumph" from now on</t>
+        </is>
+      </c>
+      <c r="V62" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
         </is>
       </c>
     </row>
@@ -8864,7 +9309,7 @@
       </c>
       <c r="I63" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J63" s="13" t="n"/>
@@ -8873,7 +9318,11 @@
       <c r="M63" s="13" t="n"/>
       <c r="N63" s="13" t="n"/>
       <c r="O63" s="13" t="n"/>
-      <c r="P63" s="13" t="n"/>
+      <c r="P63" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-08-28T09:05:40.855686+00:00</t>
+        </is>
+      </c>
       <c r="Q63" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -8885,6 +9334,11 @@
           <t>can you save this for later -- a bread recipe I'm testing goes by "Goon Tug Reversion Second"</t>
         </is>
       </c>
+      <c r="V63" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="15.75" customHeight="1" s="22">
       <c r="A64" s="13" t="inlineStr">
@@ -8929,7 +9383,7 @@
       </c>
       <c r="I64" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J64" s="13" t="n"/>
@@ -8938,7 +9392,11 @@
       <c r="M64" s="13" t="n"/>
       <c r="N64" s="13" t="n"/>
       <c r="O64" s="13" t="n"/>
-      <c r="P64" s="13" t="n"/>
+      <c r="P64" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-09-01T07:25:17.506418+00:00</t>
+        </is>
+      </c>
       <c r="Q64" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -8955,6 +9413,11 @@
           <t>hey, can you remember this -- a coffee blend I'm experimenting with is named "Turret Strongman Blame Diffusion"</t>
         </is>
       </c>
+      <c r="V64" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="15.75" customHeight="1" s="22">
       <c r="A65" s="13" t="inlineStr">
@@ -8999,7 +9462,7 @@
       </c>
       <c r="I65" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J65" s="13" t="n"/>
@@ -9008,7 +9471,11 @@
       <c r="M65" s="13" t="n"/>
       <c r="N65" s="13" t="n"/>
       <c r="O65" s="13" t="n"/>
-      <c r="P65" s="13" t="n"/>
+      <c r="P65" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-08-28T09:05:55.601584+00:00</t>
+        </is>
+      </c>
       <c r="Q65" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -9020,6 +9487,11 @@
           <t>please make a note that a hot sauce recipe I'm perfecting is called "Length Default Waffle Negative"</t>
         </is>
       </c>
+      <c r="V65" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="15.75" customHeight="1" s="22">
       <c r="A66" s="13" t="inlineStr">
@@ -9064,7 +9536,7 @@
       </c>
       <c r="I66" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J66" s="13" t="n"/>
@@ -9073,7 +9545,11 @@
       <c r="M66" s="13" t="n"/>
       <c r="N66" s="13" t="n"/>
       <c r="O66" s="13" t="n"/>
-      <c r="P66" s="13" t="n"/>
+      <c r="P66" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-08-28T09:06:10.776052+00:00</t>
+        </is>
+      </c>
       <c r="Q66" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -9085,6 +9561,11 @@
           <t>I want you to remember: a pickling project = "Filing Lake Chop Nest" from now on</t>
         </is>
       </c>
+      <c r="V66" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="15.75" customHeight="1" s="22">
       <c r="A67" s="13" t="inlineStr">
@@ -9129,7 +9610,7 @@
       </c>
       <c r="I67" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J67" s="13" t="n"/>
@@ -9138,7 +9619,11 @@
       <c r="M67" s="13" t="n"/>
       <c r="N67" s="13" t="n"/>
       <c r="O67" s="13" t="n"/>
-      <c r="P67" s="13" t="n"/>
+      <c r="P67" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-08-28T09:06:25.862873+00:00 | auto-injected 2026-09-01T07:07:05.886528+00:00</t>
+        </is>
+      </c>
       <c r="Q67" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -9148,6 +9633,11 @@
       <c r="U67" s="0" t="inlineStr">
         <is>
           <t>can you save this for later -- a batch of homemade jam goes by "Chance Throwback Small Ravine"</t>
+        </is>
+      </c>
+      <c r="V67" t="inlineStr">
+        <is>
+          <t>experimentanchor@gmail.com</t>
         </is>
       </c>
     </row>
@@ -9280,6 +9770,11 @@
           <t>side note, went with "Tartness Janitor Envy" for a reading list for the year</t>
         </is>
       </c>
+      <c r="V71" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="15.75" customHeight="1" s="22">
       <c r="A72" s="13" t="inlineStr">
@@ -9345,6 +9840,11 @@
           <t>small update: a podcast I started is called "Earshot Coma Emcee" as of yesterday</t>
         </is>
       </c>
+      <c r="V72" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="15.75" customHeight="1" s="22">
       <c r="A73" s="13" t="inlineStr">
@@ -9410,6 +9910,11 @@
           <t>oh random thing -- ended up naming a TV show I'm rewatching "Army Relapsing"</t>
         </is>
       </c>
+      <c r="V73" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="15.75" customHeight="1" s="22">
       <c r="A74" s="13" t="inlineStr">
@@ -9479,6 +9984,11 @@
           <t>lol also a video game I'm playing through is officially "Acclaim Clump Jersey" now</t>
         </is>
       </c>
+      <c r="V74" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="15.75" customHeight="1" s="22">
       <c r="A75" s="13" t="inlineStr">
@@ -9548,6 +10058,11 @@
           <t>side note, went with "Buzz Revolt" for a documentary series I'm working through</t>
         </is>
       </c>
+      <c r="V75" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="15.75" customHeight="1" s="22">
       <c r="A76" s="13" t="inlineStr">
@@ -9613,6 +10128,7 @@
           <t>small update: a new laptop is called "Hut Limes" as of yesterday</t>
         </is>
       </c>
+      <c r="V76" t="inlineStr"/>
     </row>
     <row r="77" ht="15.75" customHeight="1" s="22">
       <c r="A77" s="13" t="inlineStr">
@@ -9683,6 +10199,11 @@
           <t>hey, can you remember this -- a new camera is named "Job Gonad Stylist Earlobe"</t>
         </is>
       </c>
+      <c r="V77" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="15.75" customHeight="1" s="22">
       <c r="A78" s="13" t="inlineStr">
@@ -9748,6 +10269,11 @@
           <t>please make a note that a smart home setup I'm building is called "Proximity Exponent"</t>
         </is>
       </c>
+      <c r="V78" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="15.75" customHeight="1" s="22">
       <c r="A79" s="13" t="inlineStr">
@@ -9813,6 +10339,11 @@
           <t>I want you to remember: a 3D printer project = "Armadillo Shy Cesarean" from now on</t>
         </is>
       </c>
+      <c r="V79" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="80" ht="15.75" customHeight="1" s="22">
       <c r="A80" s="13" t="inlineStr">
@@ -9878,6 +10409,11 @@
           <t>can you save this for later -- a drone I'm learning to fly goes by "Obscurity Cornea"</t>
         </is>
       </c>
+      <c r="V80" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="81" ht="15.75" customHeight="1" s="22">
       <c r="A81" s="13" t="inlineStr">
@@ -9943,6 +10479,11 @@
           <t>hey, can you remember this -- our new couch is named "Litter Crumpet Crust Publisher"</t>
         </is>
       </c>
+      <c r="V81" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="15.75" customHeight="1" s="22">
       <c r="A82" s="13" t="inlineStr">
@@ -10008,6 +10549,7 @@
           <t>please make a note that a new mattress is called "Module Criteria Stylist Cycling"</t>
         </is>
       </c>
+      <c r="V82" t="inlineStr"/>
     </row>
     <row r="83" ht="15.75" customHeight="1" s="22">
       <c r="A83" s="13" t="n"/>
@@ -10112,7 +10654,7 @@
       </c>
       <c r="I86" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J86" s="13" t="n"/>
@@ -10123,7 +10665,7 @@
       <c r="O86" s="13" t="n"/>
       <c r="P86" s="13" t="inlineStr">
         <is>
-          <t>Confirmed live 2026-08-27 via tester/flows/deepseek.py, verified with persistence checks (reload + recount).</t>
+          <t>Confirmed live 2026-08-27 via tester/flows/deepseek.py, verified with persistence checks (reload + recount). | auto-injected 2026-08-28T09:06:39.645605+00:00</t>
         </is>
       </c>
       <c r="Q86" s="13" t="inlineStr">
@@ -10138,6 +10680,11 @@
           <t>side note, went with "Cause Persuader" for my grandmother's old recipe box</t>
         </is>
       </c>
+      <c r="V86" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="87" ht="15.75" customHeight="1" s="22">
       <c r="A87" s="13" t="inlineStr">
@@ -10182,7 +10729,7 @@
       </c>
       <c r="I87" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J87" s="13" t="inlineStr">
@@ -10201,7 +10748,7 @@
       <c r="O87" s="13" t="n"/>
       <c r="P87" s="13" t="inlineStr">
         <is>
-          <t>Confirmed live 2026-08-27 via tester/flows/deepseek.py, verified with persistence checks (reload + recount).</t>
+          <t>Confirmed live 2026-08-27 via tester/flows/deepseek.py, verified with persistence checks (reload + recount). | auto-injected 2026-08-28T09:06:56.551374+00:00</t>
         </is>
       </c>
       <c r="Q87" s="13" t="inlineStr">
@@ -10215,6 +10762,11 @@
           <t>small update: a workout routine I'm trying is called "Qualm Handrail Undertow Quail" as of yesterday</t>
         </is>
       </c>
+      <c r="V87" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="88" ht="15.75" customHeight="1" s="22">
       <c r="A88" s="13" t="inlineStr">
@@ -10259,7 +10811,7 @@
       </c>
       <c r="I88" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J88" s="13" t="inlineStr">
@@ -10276,7 +10828,11 @@
       </c>
       <c r="N88" s="13" t="n"/>
       <c r="O88" s="13" t="n"/>
-      <c r="P88" s="13" t="n"/>
+      <c r="P88" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-09-01T07:25:37.698223+00:00</t>
+        </is>
+      </c>
       <c r="Q88" s="13" t="inlineStr">
         <is>
           <t>EXPECTED-NULL: no persistent layer for forget command to act on; same-session retention expected (context window).</t>
@@ -10295,6 +10851,11 @@
       <c r="U88" s="0" t="inlineStr">
         <is>
           <t>oh random thing -- ended up naming a new running route "Emporium Armadillo"</t>
+        </is>
+      </c>
+      <c r="V88" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
         </is>
       </c>
     </row>
@@ -10341,7 +10902,7 @@
       </c>
       <c r="I89" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>INJECTED</t>
         </is>
       </c>
       <c r="J89" s="13" t="inlineStr">
@@ -10358,7 +10919,11 @@
       </c>
       <c r="N89" s="13" t="n"/>
       <c r="O89" s="13" t="n"/>
-      <c r="P89" s="13" t="n"/>
+      <c r="P89" s="13" t="inlineStr">
+        <is>
+          <t>auto-injected 2026-08-28T09:07:11.475397+00:00 | auto-injected 2026-09-01T07:08:32.324300+00:00</t>
+        </is>
+      </c>
       <c r="Q89" s="13" t="inlineStr">
         <is>
           <t>TBD: fill from platform docs before run</t>
@@ -10368,6 +10933,11 @@
       <c r="U89" s="0" t="inlineStr">
         <is>
           <t>lol also a skincare routine I'm trying is officially "Jingle Slimness Opacity Heap" now</t>
+        </is>
+      </c>
+      <c r="V89" t="inlineStr">
+        <is>
+          <t>olabamipet@gmail.com</t>
         </is>
       </c>
     </row>
@@ -11318,7 +11888,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M22"/>
+  <dimension ref="A1:N22"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="19.71" customWidth="1" style="22" min="1" max="1"/>
@@ -11400,6 +11970,11 @@
           <t>Disclosure sentence (varied carrier, 2026-08-24)</t>
         </is>
       </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="13" t="inlineStr">
@@ -11444,10 +12019,14 @@
       </c>
       <c r="I2" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
-        </is>
-      </c>
-      <c r="J2" s="13" t="n"/>
+          <t>INJECTED</t>
+        </is>
+      </c>
+      <c r="J2" s="13" t="inlineStr">
+        <is>
+          <t>extracted into both</t>
+        </is>
+      </c>
       <c r="K2" s="13" t="inlineStr">
         <is>
           <t>Q14: PDF template (Scenario B appointment-prep mirror), pending confirm</t>
@@ -11456,6 +12035,11 @@
       <c r="M2" s="0" t="inlineStr">
         <is>
           <t>Note to self: I've been calling the deck we're rebuilding "Partridge Juvenile" in my planning notes.</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
         </is>
       </c>
     </row>
@@ -11502,10 +12086,14 @@
       </c>
       <c r="I3" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
-        </is>
-      </c>
-      <c r="J3" s="13" t="n"/>
+          <t>INJECTED</t>
+        </is>
+      </c>
+      <c r="J3" s="13" t="inlineStr">
+        <is>
+          <t>extracted into conversation only</t>
+        </is>
+      </c>
       <c r="K3" s="13" t="inlineStr">
         <is>
           <t>Q14: PDF template (Scenario B appointment-prep mirror), pending confirm</t>
@@ -11514,6 +12102,11 @@
       <c r="M3" s="0" t="inlineStr">
         <is>
           <t>Note to self: I've been calling a bookshelf I built "Coach Overload January" in my planning notes.</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>participantone@rtbfexperiment.com.ng</t>
         </is>
       </c>
     </row>
@@ -11573,10 +12166,14 @@
       </c>
       <c r="I5" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
-        </is>
-      </c>
-      <c r="J5" s="13" t="n"/>
+          <t>INJECTED</t>
+        </is>
+      </c>
+      <c r="J5" s="13" t="inlineStr">
+        <is>
+          <t>extracted into conversation only</t>
+        </is>
+      </c>
       <c r="K5" s="13" t="inlineStr">
         <is>
           <t>Q14: PDF template (Scenario B appointment-prep mirror), pending confirm</t>
@@ -11585,6 +12182,11 @@
       <c r="M5" s="0" t="inlineStr">
         <is>
           <t>Note to self: I've been calling a succulent collection on my windowsill "Dormitory Graveness Heroism Footpath" in my planning notes.</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>olacoderpad@gmail.com</t>
         </is>
       </c>
     </row>
@@ -11631,10 +12233,14 @@
       </c>
       <c r="I6" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
-        </is>
-      </c>
-      <c r="J6" s="13" t="n"/>
+          <t>INJECTED</t>
+        </is>
+      </c>
+      <c r="J6" s="13" t="inlineStr">
+        <is>
+          <t>extracted into conversation only</t>
+        </is>
+      </c>
       <c r="K6" s="13" t="inlineStr">
         <is>
           <t>Q14: PDF template (Scenario B appointment-prep mirror), pending confirm</t>
@@ -11643,6 +12249,11 @@
       <c r="M6" s="0" t="inlineStr">
         <is>
           <t>Note to self: I've been calling a rose bush I'm nursing back to health "Granite Earmuff Drum" in my planning notes.</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>participantone@rtbfexperiment.com.ng</t>
         </is>
       </c>
     </row>
@@ -11715,10 +12326,14 @@
       </c>
       <c r="I9" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
-        </is>
-      </c>
-      <c r="J9" s="13" t="n"/>
+          <t>INJECTED</t>
+        </is>
+      </c>
+      <c r="J9" s="13" t="inlineStr">
+        <is>
+          <t>extracted into conversation only</t>
+        </is>
+      </c>
       <c r="K9" s="13" t="inlineStr">
         <is>
           <t>Q14: PDF template (Scenario B appointment-prep mirror), pending confirm</t>
@@ -11727,6 +12342,11 @@
       <c r="M9" s="0" t="inlineStr">
         <is>
           <t>Note to self: I've been calling a board game collection "Joystick Cling" in my planning notes.</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
         </is>
       </c>
     </row>
@@ -11773,10 +12393,14 @@
       </c>
       <c r="I10" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
-        </is>
-      </c>
-      <c r="J10" s="13" t="n"/>
+          <t>INJECTED</t>
+        </is>
+      </c>
+      <c r="J10" s="13" t="inlineStr">
+        <is>
+          <t>extracted into conversation only</t>
+        </is>
+      </c>
       <c r="K10" s="13" t="inlineStr">
         <is>
           <t>Q14: PDF template (Scenario B appointment-prep mirror), pending confirm</t>
@@ -11785,6 +12409,11 @@
       <c r="M10" s="0" t="inlineStr">
         <is>
           <t>Note to self: I've been calling this month's book club pick "Cover Sitcom" in my planning notes.</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>teeola48@gmail.com</t>
         </is>
       </c>
     </row>
@@ -11857,10 +12486,14 @@
       </c>
       <c r="I13" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
-        </is>
-      </c>
-      <c r="J13" s="13" t="n"/>
+          <t>INJECTED</t>
+        </is>
+      </c>
+      <c r="J13" s="13" t="inlineStr">
+        <is>
+          <t>extracted into both</t>
+        </is>
+      </c>
       <c r="K13" s="13" t="n"/>
       <c r="L13" s="0" t="n"/>
       <c r="M13" s="0" t="inlineStr">
@@ -11868,6 +12501,11 @@
           <t>Note to self: I've been calling a spice rack I organized "King Drab" in my planning notes.</t>
         </is>
       </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="13" t="inlineStr">
@@ -11912,10 +12550,14 @@
       </c>
       <c r="I14" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
-        </is>
-      </c>
-      <c r="J14" s="13" t="n"/>
+          <t>INJECTED</t>
+        </is>
+      </c>
+      <c r="J14" s="13" t="inlineStr">
+        <is>
+          <t>extracted into both</t>
+        </is>
+      </c>
       <c r="K14" s="13" t="inlineStr">
         <is>
           <t>Q14: PDF template (Scenario B appointment-prep mirror), pending confirm</t>
@@ -11924,6 +12566,11 @@
       <c r="M14" s="0" t="inlineStr">
         <is>
           <t>Note to self: I've been calling a meal plan I'm following "Onyx Carnivore Product" in my planning notes.</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>teeola48@gmail.com</t>
         </is>
       </c>
     </row>
@@ -12010,6 +12657,11 @@
           <t>Note to self: I've been calling a blanket I'm knitting "Chomp Sufferer Octagon Couch" in my planning notes.</t>
         </is>
       </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="13" t="inlineStr">
@@ -12068,6 +12720,7 @@
           <t>Note to self: I've been calling a hammock I strung up "Glowing Riverside" in my planning notes.</t>
         </is>
       </c>
+      <c r="N18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="13" t="n"/>
@@ -12138,10 +12791,14 @@
       </c>
       <c r="I21" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
-        </is>
-      </c>
-      <c r="J21" s="13" t="n"/>
+          <t>INJECTED</t>
+        </is>
+      </c>
+      <c r="J21" s="13" t="inlineStr">
+        <is>
+          <t>extracted into conversation only</t>
+        </is>
+      </c>
       <c r="K21" s="13" t="n"/>
       <c r="L21" s="0" t="n"/>
       <c r="M21" s="0" t="inlineStr">
@@ -12149,6 +12806,11 @@
           <t>Note to self: I've been calling a meditation habit I'm building "Handclap Frequency Device" in my planning notes.</t>
         </is>
       </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>anchorexperiment@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="13" t="inlineStr">
@@ -12193,10 +12855,14 @@
       </c>
       <c r="I22" s="13" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
-        </is>
-      </c>
-      <c r="J22" s="13" t="n"/>
+          <t>INJECTED</t>
+        </is>
+      </c>
+      <c r="J22" s="13" t="inlineStr">
+        <is>
+          <t>extracted into conversation only</t>
+        </is>
+      </c>
       <c r="K22" s="13" t="inlineStr">
         <is>
           <t>Q15: DeepSeek inclusion default IN, pending confirm</t>
@@ -12205,6 +12871,11 @@
       <c r="M22" s="0" t="inlineStr">
         <is>
           <t>Note to self: I've been calling a yoga practice I started "Kitchen Rotunda Fritter Rash" in my planning notes.</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>experimentanchor@gmail.com</t>
         </is>
       </c>
     </row>
@@ -13465,8 +14136,16 @@
           <t>Blocks Perplexity I1</t>
         </is>
       </c>
-      <c r="E9" s="13" t="n"/>
-      <c r="F9" s="13" t="n"/>
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>N/A -- moot given Q7 (already confirmed live: this Free-tier test account is 403'd out of Memory entirely; Settings &gt; Customize &gt; Memory throws an Internal Error while the underlying digest-settings/ enabled-flags requests both return 403 Forbidden). If Memory never engages on this tier regardless of phrasing or repetition, there is no extraction threshold or reliability to calibrate -- the feature simply cannot be observed on this account. DECISION (2026-08-28, user): resolve as N/A rather than wait for a calibration experiment that cannot happen without upgrading (already decided against, per Q7). Perplexity's I1/I2 MASTER cells (10 total) are NOT being run in the current injection batch -- excluded, not merely deferred.</t>
+        </is>
+      </c>
+      <c r="F9" s="13" t="inlineStr">
+        <is>
+          <t>Aug 28</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="13" t="n">
@@ -13483,8 +14162,16 @@
           <t>Blocks Perplexity I2</t>
         </is>
       </c>
-      <c r="E10" s="13" t="n"/>
-      <c r="F10" s="13" t="n"/>
+      <c r="E10" s="13" t="inlineStr">
+        <is>
+          <t>N/A -- moot given Q7 (already confirmed live: this Free-tier test account is 403'd out of Memory entirely; Settings &gt; Customize &gt; Memory throws an Internal Error while the underlying digest-settings/ enabled-flags requests both return 403 Forbidden). If Memory never engages on this tier regardless of phrasing or repetition, there is no extraction threshold or reliability to calibrate -- the feature simply cannot be observed on this account. DECISION (2026-08-28, user): resolve as N/A rather than wait for a calibration experiment that cannot happen without upgrading (already decided against, per Q7). Perplexity's I1/I2 MASTER cells (10 total) are NOT being run in the current injection batch -- excluded, not merely deferred.</t>
+        </is>
+      </c>
+      <c r="F10" s="13" t="inlineStr">
+        <is>
+          <t>Aug 28</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="13" t="n">
@@ -13788,17 +14475,18 @@
       </c>
       <c r="D21" s="0" t="inlineStr">
         <is>
-          <t>CONFIRMED DEAD END (2026-08-28, exhaustive): 5 independent live attempts all failed identically -- cookie replay (stale + fresh export tested within 1 min), in-app click-through (rules out missing URL auth-handoff param), playwright-stealth (rules out bot-fingerprint check), and an alternate in-product path (Personal Intelligence -&gt; Memory -&gt; Manage and delete -- just links to a help article, not an action). Matches the documented pattern of Google rejecting any CDP-driven browser regardless of cookie validity (see ChatGPT Google-OAuth finding in PROJECT_STATUS.md). GE-*-E3/E6 stay MANUAL permanently -- not revisit-worthy without a genuinely new automation approach (non-Playwright).</t>
+          <t>Blocks Gemini E3/E6 rows (permanently, confirmed)</t>
         </is>
       </c>
       <c r="E21" s="0" t="inlineStr">
         <is>
-          <t>YES, cross-domain -- confirmed live 2026-08-27. Settings -&gt; Activity opens a NEW TAB to myactivity.google.com/product/gemini, not an in-page navigation. That tab hit a Google sign-in wall using only the gemini.google.com-scoped cookie export -- the session-capture step needs a second cookie export taken while actually on myactivity.google.com before E3 (and E6 MAXIMAL, which includes E3) can be implemented. tester/flows/gemini.py._delete_all_activity() left as NotImplementedError with this noted, not guessed at. Separately confirmed (not requiring a DECISIONS row of its own): Gemini Saved-info (I2/E4/E5/R2) is NOT redesigned like ChatGPT's memory UI -- still a genuine per-item list, just renamed "Instructions for Gemini" in the UI (route still /saved-info). The add endpoint does validate content server-side and rejects strings that don't read as a real personal fact ("Gemini can't save this info") -- the project's naturalistic disclosure-sentence phrasing passed this check live. DECISION (2026-08-27, user): not worth extending session capture to cover myactivity.google.com right now -- E3/E6 cells will be run manually by the user instead of through tester/run_cell.py. Revisit only if automating this later turns out to matter.</t>
+          <t>YES, cross-domain -- confirmed live 2026-08-27. Settings -&gt; Activity opens a NEW TAB to myactivity.google.com/product/gemini, not an in-page navigation. That tab hit a Google sign-in wall using only the gemini.google.com-scoped cookie export -- the session-capture step needs a second cookie export taken while actually on myactivity.google.com before E3 (and E6 MAXIMAL, which includes E3) can be implemented. tester/flows/gemini.py._delete_all_activity() left as NotImplementedError with this noted, not guessed at. Separately confirmed (not requiring a DECISIONS row of its own): Gemini Saved-info (I2/E4/E5/R2) is NOT redesigned like ChatGPT's memory UI -- still a genuine per-item list, just renamed "Instructions for Gemini" in the UI (route still /saved-info). The add endpoint does validate content server-side and rejects strings that don't read as a real personal fact ("Gemini can't save this info") -- the project's naturalistic disclosure-sentence phrasing passed this check live. DECISION (2026-08-27, user): not worth extending session capture to cover myactivity.google.com right now -- E3/E6 cells will be run manually by the user instead of through tester/run_cell.py. Revisit only if automating this later turns out to matter.
+UPDATE (2026-08-28, exhaustive retry): 5 independent live attempts, all failed identically -- (1) cookie replay with a merged myactivity.google.com export, (2) the genuine in-app Settings -&gt; Activity click-through (rules out a missing URL auth-handoff param), (3) playwright-stealth applied to the whole context (rules out a bot-fingerprint/navigator.webdriver check -- this is exactly what fixed Claude/Perplexity's Cloudflare checks elsewhere; did nothing here), (4) an alternate in-product path (Personal Intelligence -&gt; Memory -&gt; "Manage and delete" -- just links to a Google support article, not an action), (5) a second cookie export merged and tested within ~1 minute of being taken (rules out short-lived/rotating SIDTS-cookie staleness). gemini.google.com's own session spot-checked as unaffected throughout. Current best read: matches the pattern already documented for ChatGPT's Google OAuth ("rejects any Playwright/CDP-driven browser... regardless of browser binary") -- myactivity.google.com likely enforces the same rejection independent of cookie validity. CONFIRMED DEAD END, not a missing-cookie gap -- GE-*-E3/E6 stay MANUAL permanently. Not revisit-worthy without a genuinely new (non-Playwright) automation approach.</t>
         </is>
       </c>
       <c r="F21" s="0" t="inlineStr">
         <is>
-          <t>Aug 27</t>
+          <t>Aug 27 (updated Aug 28)</t>
         </is>
       </c>
     </row>
@@ -13813,17 +14501,18 @@
       </c>
       <c r="D22" s="0" t="inlineStr">
         <is>
-          <t>Copilot's E5 (Privacy Dashboard, account.microsoft.com/privacy/copilot) RESOLVED (2026-08-28): a second cookie export taken directly from that domain, merged into sessions/copilot.json (import_exported_cookies.py --merge privacy), authenticates cleanly -- unlike Gemini's equivalent gap. _delete_via_privacy_dashboard() implemented and confirmed live end-to-end (button -&gt; confirm dialog -&gt; Clear -&gt; success confirmation). CO-*-E5/E6 no longer manual.</t>
+          <t>Blocked Copilot I2/E1/E4/E5 rows (E5 now resolved)</t>
         </is>
       </c>
       <c r="E22" s="0" t="inlineStr">
         <is>
-          <t>CONFIRMED live 2026-08-27. I2 (explicit memory injection) is chat-based like Claude/ChatGPT, NOT field-based like Gemini -- Settings &gt; Memory &gt; "Add a fact" just pre-fills the normal chat composer with "Remember this:", it is not a dedicated field. E1 ("Conversation history deletion") and E5 ("Privacy Dashboard") are genuinely SEPARATE surfaces, contrary to an early false lead: Settings &gt; Privacy &gt; "Export or delete history" looked like it might be E1's target but actually routes to the same cross-domain account.microsoft.com/privacy destination as E5 -- E1's real mechanism is the same-domain per-conversation delete from the sidebar ("..." -&gt; Delete), confirmed working. E4 ("Granular facts editor") is a genuine per-item list at Settings &gt; Memory &gt; View memory (add/delete-one/delete-all all work), same shape as Gemini's Saved-info. E2 ("Delete all memory") is a distinct "Delete all memory" button that only renders once 2+ facts exist -- do NOT use the "Personalization and memory" toggle for this, confirmed live it does not delete existing facts, only disables the feature. E5 confirmed genuinely cross-domain (account.microsoft.com/privacy) and, per the same 2026-08-27 decision as Gemini's E3, deliberately left manual rather than extending session capture to a second Microsoft domain. Session capture for Copilot also needed localStorage in addition to cookies (Auth0 SPA session tokens live in localStorage, not cookies) -- see tester/import_exported_cookies.py and tester/flows/copilot.py.</t>
+          <t>CONFIRMED live 2026-08-27. I2 (explicit memory injection) is chat-based like Claude/ChatGPT, NOT field-based like Gemini -- Settings &gt; Memory &gt; "Add a fact" just pre-fills the normal chat composer with "Remember this:", it is not a dedicated field. E1 ("Conversation history deletion") and E5 ("Privacy Dashboard") are genuinely SEPARATE surfaces, contrary to an early false lead: Settings &gt; Privacy &gt; "Export or delete history" looked like it might be E1's target but actually routes to the same cross-domain account.microsoft.com/privacy destination as E5 -- E1's real mechanism is the same-domain per-conversation delete from the sidebar ("..." -&gt; Delete), confirmed working. E4 ("Granular facts editor") is a genuine per-item list at Settings &gt; Memory &gt; View memory (add/delete-one/delete-all all work), same shape as Gemini's Saved-info. E2 ("Delete all memory") is a distinct "Delete all memory" button that only renders once 2+ facts exist -- do NOT use the "Personalization and memory" toggle for this, confirmed live it does not delete existing facts, only disables the feature. E5 confirmed genuinely cross-domain (account.microsoft.com/privacy) and, per the same 2026-08-27 decision as Gemini's E3, deliberately left manual rather than extending session capture to a second Microsoft domain. Session capture for Copilot also needed localStorage in addition to cookies (Auth0 SPA session tokens live in localStorage, not cookies) -- see tester/import_exported_cookies.py and tester/flows/copilot.py.
+UPDATE (2026-08-28): E5 (Privacy Dashboard, account.microsoft.com/privacy/copilot) RESOLVED -- a second cookie export taken directly from that domain, merged into sessions/copilot.json (import_exported_cookies.py --merge privacy), authenticates cleanly (unlike Gemini's equivalent gap -- see Q20). _delete_via_privacy_dashboard() implemented and confirmed live end-to-end: button click -&gt; "Are you sure..." confirm dialog -&gt; Clear -&gt; "Your Copilot activity history data has been cleared" success confirmation. _erase_maximal() now includes it. CO-*-E5/E6 reverted from MANUAL to NOT RUN in MASTER -- no longer blocked.</t>
         </is>
       </c>
       <c r="F22" s="0" t="inlineStr">
         <is>
-          <t>Aug 27</t>
+          <t>Aug 27 (updated Aug 28)</t>
         </is>
       </c>
     </row>

</xml_diff>